<commit_message>
Add 9 knowledge-layer trading rules from trading-knowledge research
Fear&Greed contrarian nudge, min reward:risk gate, kill switch, hard
daily loss limit, ATR-scaled TP legs, 24h trend alignment filter, VWAP
deviation gate, OBV divergence detection, VADER->FinBERT sentiment
upgrade. Applied to both spot-long and futures-short paths.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/leverage_journal.xlsx
+++ b/leverage_journal.xlsx
@@ -459,7 +459,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>300.99</v>
+        <v>231.86</v>
       </c>
       <c r="C2" t="n">
         <v>50</v>
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1874.28</v>
+        <v>1750.95</v>
       </c>
       <c r="C3" t="n">
         <v>50</v>
@@ -489,7 +489,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4125.15</v>
+        <v>3919.62</v>
       </c>
       <c r="C4" t="n">
         <v>50</v>
@@ -505,7 +505,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>21432.13</v>
+        <v>21021.1</v>
       </c>
       <c r="C5" t="n">
         <v>50</v>
@@ -521,7 +521,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1923.51</v>
+        <v>2109.3</v>
       </c>
       <c r="C6" t="n">
         <v>50</v>
@@ -535,7 +535,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-902.91</v>
+        <v>-695.52</v>
       </c>
       <c r="C7" t="n">
         <v>50</v>
@@ -551,7 +551,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-1412.1</v>
+        <v>-1066.46</v>
       </c>
       <c r="C8" t="n">
         <v>50</v>
@@ -567,7 +567,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>7140.9</v>
+        <v>7832.15</v>
       </c>
       <c r="C9" t="n">
         <v>50</v>
@@ -713,7 +713,7 @@
         <v>1.589</v>
       </c>
       <c r="F2" t="n">
-        <v>1.447</v>
+        <v>1.462</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -725,30 +725,30 @@
         <v>20.04</v>
       </c>
       <c r="J2" t="n">
-        <v>-8.94</v>
+        <v>-7.99</v>
       </c>
       <c r="K2" t="n">
-        <v>-1.79</v>
+        <v>-1.6</v>
       </c>
       <c r="L2" t="n">
-        <v>-26.81</v>
+        <v>-23.98</v>
       </c>
       <c r="M2" t="n">
-        <v>-5.37</v>
+        <v>-4.8</v>
       </c>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="n">
-        <v>-44.68</v>
+        <v>-39.96</v>
       </c>
       <c r="P2" t="n">
-        <v>-8.949999999999999</v>
+        <v>-8.01</v>
       </c>
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="n">
-        <v>-89.36</v>
+        <v>-79.92</v>
       </c>
       <c r="S2" t="n">
-        <v>-17.91</v>
+        <v>-16.01</v>
       </c>
       <c r="T2" t="inlineStr"/>
     </row>
@@ -773,7 +773,7 @@
         <v>1.588</v>
       </c>
       <c r="F3" t="n">
-        <v>1.447</v>
+        <v>1.462</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -785,30 +785,30 @@
         <v>19.99</v>
       </c>
       <c r="J3" t="n">
-        <v>-8.880000000000001</v>
+        <v>-7.93</v>
       </c>
       <c r="K3" t="n">
-        <v>-1.77</v>
+        <v>-1.59</v>
       </c>
       <c r="L3" t="n">
-        <v>-26.64</v>
+        <v>-23.8</v>
       </c>
       <c r="M3" t="n">
-        <v>-5.32</v>
+        <v>-4.76</v>
       </c>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="n">
-        <v>-44.4</v>
+        <v>-39.67</v>
       </c>
       <c r="P3" t="n">
-        <v>-8.869999999999999</v>
+        <v>-7.93</v>
       </c>
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="n">
-        <v>-88.79000000000001</v>
+        <v>-79.34999999999999</v>
       </c>
       <c r="S3" t="n">
-        <v>-17.75</v>
+        <v>-15.86</v>
       </c>
       <c r="T3" t="inlineStr"/>
     </row>
@@ -833,7 +833,7 @@
         <v>1.59</v>
       </c>
       <c r="F4" t="n">
-        <v>1.447</v>
+        <v>1.462</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -845,30 +845,30 @@
         <v>20.01</v>
       </c>
       <c r="J4" t="n">
-        <v>-8.99</v>
+        <v>-8.050000000000001</v>
       </c>
       <c r="K4" t="n">
-        <v>-1.8</v>
+        <v>-1.61</v>
       </c>
       <c r="L4" t="n">
-        <v>-26.98</v>
+        <v>-24.15</v>
       </c>
       <c r="M4" t="n">
-        <v>-5.4</v>
+        <v>-4.83</v>
       </c>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="n">
-        <v>-44.97</v>
+        <v>-40.25</v>
       </c>
       <c r="P4" t="n">
-        <v>-9</v>
+        <v>-8.06</v>
       </c>
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="n">
-        <v>-89.94</v>
+        <v>-80.5</v>
       </c>
       <c r="S4" t="n">
-        <v>-18</v>
+        <v>-16.11</v>
       </c>
       <c r="T4" t="inlineStr"/>
     </row>
@@ -1081,7 +1081,7 @@
         <v>0.10701</v>
       </c>
       <c r="F8" t="n">
-        <v>0.07554</v>
+        <v>0.07357</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -1093,16 +1093,16 @@
         <v>0.11</v>
       </c>
       <c r="J8" t="n">
-        <v>-29.41</v>
+        <v>-31.25</v>
       </c>
       <c r="K8" t="n">
         <v>-0.03</v>
       </c>
       <c r="L8" t="n">
-        <v>-88.23</v>
+        <v>-93.75</v>
       </c>
       <c r="M8" t="n">
-        <v>-0.09</v>
+        <v>-0.1</v>
       </c>
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="n">
@@ -1621,7 +1621,7 @@
         <v>0.002129</v>
       </c>
       <c r="F16" t="n">
-        <v>0.001958</v>
+        <v>0.001969</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -1633,30 +1633,30 @@
         <v>102.52</v>
       </c>
       <c r="J16" t="n">
-        <v>-8.029999999999999</v>
+        <v>-7.52</v>
       </c>
       <c r="K16" t="n">
-        <v>-8.23</v>
+        <v>-7.7</v>
       </c>
       <c r="L16" t="n">
-        <v>-24.1</v>
+        <v>-22.55</v>
       </c>
       <c r="M16" t="n">
-        <v>-24.7</v>
+        <v>-23.11</v>
       </c>
       <c r="N16" t="inlineStr"/>
       <c r="O16" t="n">
-        <v>-40.16</v>
+        <v>-37.58</v>
       </c>
       <c r="P16" t="n">
-        <v>-41.17</v>
+        <v>-38.52</v>
       </c>
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="n">
-        <v>-80.31999999999999</v>
+        <v>-75.15000000000001</v>
       </c>
       <c r="S16" t="n">
-        <v>-82.34</v>
+        <v>-77.05</v>
       </c>
       <c r="T16" t="inlineStr"/>
     </row>
@@ -2009,7 +2009,7 @@
         <v>2.68</v>
       </c>
       <c r="F22" t="n">
-        <v>2.531</v>
+        <v>2.495</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -2021,30 +2021,30 @@
         <v>5.87</v>
       </c>
       <c r="J22" t="n">
-        <v>-5.56</v>
+        <v>-6.9</v>
       </c>
       <c r="K22" t="n">
-        <v>-0.33</v>
+        <v>-0.41</v>
       </c>
       <c r="L22" t="n">
-        <v>-16.68</v>
+        <v>-20.71</v>
       </c>
       <c r="M22" t="n">
-        <v>-0.98</v>
+        <v>-1.22</v>
       </c>
       <c r="N22" t="inlineStr"/>
       <c r="O22" t="n">
-        <v>-27.8</v>
+        <v>-34.51</v>
       </c>
       <c r="P22" t="n">
-        <v>-1.63</v>
+        <v>-2.03</v>
       </c>
       <c r="Q22" t="inlineStr"/>
       <c r="R22" t="n">
-        <v>-55.6</v>
+        <v>-69.03</v>
       </c>
       <c r="S22" t="n">
-        <v>-3.26</v>
+        <v>-4.05</v>
       </c>
       <c r="T22" t="inlineStr"/>
     </row>
@@ -3545,7 +3545,7 @@
         <v>0.1769</v>
       </c>
       <c r="F46" t="n">
-        <v>0.0798</v>
+        <v>0.0765</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -3557,10 +3557,10 @@
         <v>1502.06</v>
       </c>
       <c r="J46" t="n">
-        <v>-54.89</v>
+        <v>-56.76</v>
       </c>
       <c r="K46" t="n">
-        <v>-824.48</v>
+        <v>-852.5</v>
       </c>
       <c r="L46" t="n">
         <v>-100</v>
@@ -3617,7 +3617,7 @@
         <v>0.1668545406313555</v>
       </c>
       <c r="F47" t="n">
-        <v>0.1627</v>
+        <v>0.1623</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -3629,30 +3629,30 @@
         <v>2264.35</v>
       </c>
       <c r="J47" t="n">
-        <v>-2.49</v>
+        <v>-2.73</v>
       </c>
       <c r="K47" t="n">
-        <v>-56.38</v>
+        <v>-61.81</v>
       </c>
       <c r="L47" t="n">
-        <v>-7.47</v>
+        <v>-8.19</v>
       </c>
       <c r="M47" t="n">
-        <v>-169.14</v>
+        <v>-185.43</v>
       </c>
       <c r="N47" t="inlineStr"/>
       <c r="O47" t="n">
-        <v>-12.45</v>
+        <v>-13.65</v>
       </c>
       <c r="P47" t="n">
-        <v>-281.9</v>
+        <v>-309.04</v>
       </c>
       <c r="Q47" t="inlineStr"/>
       <c r="R47" t="n">
-        <v>-24.9</v>
+        <v>-27.3</v>
       </c>
       <c r="S47" t="n">
-        <v>-563.8</v>
+        <v>-618.09</v>
       </c>
       <c r="T47" t="inlineStr"/>
     </row>
@@ -3869,7 +3869,7 @@
         <v>0.0675</v>
       </c>
       <c r="F51" t="n">
-        <v>0.0672</v>
+        <v>0.06610000000000001</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -3881,30 +3881,30 @@
         <v>2251.56</v>
       </c>
       <c r="J51" t="n">
-        <v>-0.44</v>
+        <v>-2.07</v>
       </c>
       <c r="K51" t="n">
-        <v>-10.01</v>
+        <v>-46.7</v>
       </c>
       <c r="L51" t="n">
-        <v>-1.33</v>
+        <v>-6.22</v>
       </c>
       <c r="M51" t="n">
-        <v>-30.02</v>
+        <v>-140.1</v>
       </c>
       <c r="N51" t="inlineStr"/>
       <c r="O51" t="n">
-        <v>-2.22</v>
+        <v>-10.37</v>
       </c>
       <c r="P51" t="n">
-        <v>-50.03</v>
+        <v>-233.49</v>
       </c>
       <c r="Q51" t="inlineStr"/>
       <c r="R51" t="n">
-        <v>-4.44</v>
+        <v>-20.74</v>
       </c>
       <c r="S51" t="n">
-        <v>-100.07</v>
+        <v>-466.99</v>
       </c>
       <c r="T51" t="inlineStr"/>
     </row>
@@ -4162,7 +4162,7 @@
         <v>12.61</v>
       </c>
       <c r="E2" t="n">
-        <v>1.447</v>
+        <v>1.462</v>
       </c>
       <c r="F2" t="n">
         <v>1.589</v>
@@ -4177,30 +4177,30 @@
         <v>20.04</v>
       </c>
       <c r="J2" t="n">
-        <v>9.81</v>
+        <v>8.69</v>
       </c>
       <c r="K2" t="n">
-        <v>1.97</v>
+        <v>1.74</v>
       </c>
       <c r="L2" t="n">
-        <v>26.81</v>
+        <v>23.98</v>
       </c>
       <c r="M2" t="n">
-        <v>5.37</v>
+        <v>4.8</v>
       </c>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="n">
-        <v>44.68</v>
+        <v>39.96</v>
       </c>
       <c r="P2" t="n">
-        <v>8.949999999999999</v>
+        <v>8.01</v>
       </c>
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="n">
-        <v>89.36</v>
+        <v>79.92</v>
       </c>
       <c r="S2" t="n">
-        <v>17.91</v>
+        <v>16.01</v>
       </c>
       <c r="T2" t="inlineStr"/>
     </row>
@@ -4222,7 +4222,7 @@
         <v>12.586</v>
       </c>
       <c r="E3" t="n">
-        <v>1.447</v>
+        <v>1.462</v>
       </c>
       <c r="F3" t="n">
         <v>1.588</v>
@@ -4237,30 +4237,30 @@
         <v>19.99</v>
       </c>
       <c r="J3" t="n">
-        <v>9.74</v>
+        <v>8.619999999999999</v>
       </c>
       <c r="K3" t="n">
-        <v>1.95</v>
+        <v>1.72</v>
       </c>
       <c r="L3" t="n">
-        <v>26.64</v>
+        <v>23.8</v>
       </c>
       <c r="M3" t="n">
-        <v>5.32</v>
+        <v>4.76</v>
       </c>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="n">
-        <v>44.4</v>
+        <v>39.67</v>
       </c>
       <c r="P3" t="n">
-        <v>8.869999999999999</v>
+        <v>7.93</v>
       </c>
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="n">
-        <v>88.79000000000001</v>
+        <v>79.34999999999999</v>
       </c>
       <c r="S3" t="n">
-        <v>17.75</v>
+        <v>15.86</v>
       </c>
       <c r="T3" t="inlineStr"/>
     </row>
@@ -4282,7 +4282,7 @@
         <v>12.586</v>
       </c>
       <c r="E4" t="n">
-        <v>1.447</v>
+        <v>1.462</v>
       </c>
       <c r="F4" t="n">
         <v>1.59</v>
@@ -4297,30 +4297,30 @@
         <v>20.01</v>
       </c>
       <c r="J4" t="n">
-        <v>9.880000000000001</v>
+        <v>8.76</v>
       </c>
       <c r="K4" t="n">
-        <v>1.98</v>
+        <v>1.75</v>
       </c>
       <c r="L4" t="n">
-        <v>26.98</v>
+        <v>24.15</v>
       </c>
       <c r="M4" t="n">
-        <v>5.4</v>
+        <v>4.83</v>
       </c>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="n">
-        <v>44.97</v>
+        <v>40.25</v>
       </c>
       <c r="P4" t="n">
-        <v>9</v>
+        <v>8.06</v>
       </c>
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="n">
-        <v>89.94</v>
+        <v>80.5</v>
       </c>
       <c r="S4" t="n">
-        <v>18</v>
+        <v>16.11</v>
       </c>
       <c r="T4" t="inlineStr"/>
     </row>
@@ -4542,7 +4542,7 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>0.07554</v>
+        <v>0.07357</v>
       </c>
       <c r="F8" t="n">
         <v>0.10701</v>
@@ -4557,30 +4557,30 @@
         <v>0.11</v>
       </c>
       <c r="J8" t="n">
-        <v>41.66</v>
+        <v>45.45</v>
       </c>
       <c r="K8" t="n">
-        <v>0.04</v>
+        <v>0.05</v>
       </c>
       <c r="L8" t="n">
-        <v>88.23</v>
+        <v>93.75</v>
       </c>
       <c r="M8" t="n">
-        <v>0.09</v>
+        <v>0.1</v>
       </c>
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="n">
-        <v>147.04</v>
+        <v>156.25</v>
       </c>
       <c r="P8" t="n">
-        <v>0.16</v>
+        <v>0.17</v>
       </c>
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="n">
-        <v>294.08</v>
+        <v>312.49</v>
       </c>
       <c r="S8" t="n">
-        <v>0.31</v>
+        <v>0.33</v>
       </c>
       <c r="T8" t="inlineStr"/>
     </row>
@@ -5050,7 +5050,7 @@
         <v>48154</v>
       </c>
       <c r="E16" t="n">
-        <v>0.001958</v>
+        <v>0.001969</v>
       </c>
       <c r="F16" t="n">
         <v>0.002129</v>
@@ -5065,30 +5065,30 @@
         <v>102.52</v>
       </c>
       <c r="J16" t="n">
-        <v>8.73</v>
+        <v>8.130000000000001</v>
       </c>
       <c r="K16" t="n">
-        <v>8.949999999999999</v>
+        <v>8.33</v>
       </c>
       <c r="L16" t="n">
-        <v>24.1</v>
+        <v>22.55</v>
       </c>
       <c r="M16" t="n">
-        <v>24.7</v>
+        <v>23.11</v>
       </c>
       <c r="N16" t="inlineStr"/>
       <c r="O16" t="n">
-        <v>40.16</v>
+        <v>37.58</v>
       </c>
       <c r="P16" t="n">
-        <v>41.17</v>
+        <v>38.52</v>
       </c>
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="n">
-        <v>80.31999999999999</v>
+        <v>75.15000000000001</v>
       </c>
       <c r="S16" t="n">
-        <v>82.34</v>
+        <v>77.05</v>
       </c>
       <c r="T16" t="inlineStr"/>
     </row>
@@ -5446,7 +5446,7 @@
         <v>2.19</v>
       </c>
       <c r="E22" t="n">
-        <v>2.531</v>
+        <v>2.495</v>
       </c>
       <c r="F22" t="n">
         <v>2.68</v>
@@ -5461,30 +5461,30 @@
         <v>5.87</v>
       </c>
       <c r="J22" t="n">
-        <v>5.89</v>
+        <v>7.41</v>
       </c>
       <c r="K22" t="n">
-        <v>0.35</v>
+        <v>0.44</v>
       </c>
       <c r="L22" t="n">
-        <v>16.68</v>
+        <v>20.71</v>
       </c>
       <c r="M22" t="n">
-        <v>0.98</v>
+        <v>1.22</v>
       </c>
       <c r="N22" t="inlineStr"/>
       <c r="O22" t="n">
-        <v>27.8</v>
+        <v>34.51</v>
       </c>
       <c r="P22" t="n">
-        <v>1.63</v>
+        <v>2.03</v>
       </c>
       <c r="Q22" t="inlineStr"/>
       <c r="R22" t="n">
-        <v>55.6</v>
+        <v>69.03</v>
       </c>
       <c r="S22" t="n">
-        <v>3.26</v>
+        <v>4.05</v>
       </c>
       <c r="T22" t="inlineStr"/>
     </row>
@@ -6994,7 +6994,7 @@
         <v>8491</v>
       </c>
       <c r="E46" t="n">
-        <v>0.0798</v>
+        <v>0.0765</v>
       </c>
       <c r="F46" t="n">
         <v>0.1769</v>
@@ -7009,30 +7009,30 @@
         <v>1502.06</v>
       </c>
       <c r="J46" t="n">
-        <v>121.68</v>
+        <v>131.24</v>
       </c>
       <c r="K46" t="n">
-        <v>1827.69</v>
+        <v>1971.33</v>
       </c>
       <c r="L46" t="n">
-        <v>164.67</v>
+        <v>170.27</v>
       </c>
       <c r="M46" t="n">
-        <v>2473.43</v>
+        <v>2557.49</v>
       </c>
       <c r="N46" t="inlineStr"/>
       <c r="O46" t="n">
-        <v>274.45</v>
+        <v>283.78</v>
       </c>
       <c r="P46" t="n">
-        <v>4122.38</v>
+        <v>4262.48</v>
       </c>
       <c r="Q46" t="inlineStr"/>
       <c r="R46" t="n">
-        <v>548.9</v>
+        <v>567.55</v>
       </c>
       <c r="S46" t="n">
-        <v>8244.76</v>
+        <v>8524.959999999999</v>
       </c>
       <c r="T46" t="inlineStr"/>
     </row>
@@ -7054,7 +7054,7 @@
         <v>13570.8</v>
       </c>
       <c r="E47" t="n">
-        <v>0.1627</v>
+        <v>0.1623</v>
       </c>
       <c r="F47" t="n">
         <v>0.1668545406313555</v>
@@ -7069,30 +7069,30 @@
         <v>2264.35</v>
       </c>
       <c r="J47" t="n">
-        <v>2.55</v>
+        <v>2.81</v>
       </c>
       <c r="K47" t="n">
-        <v>57.82</v>
+        <v>63.54</v>
       </c>
       <c r="L47" t="n">
-        <v>7.47</v>
+        <v>8.19</v>
       </c>
       <c r="M47" t="n">
-        <v>169.14</v>
+        <v>185.43</v>
       </c>
       <c r="N47" t="inlineStr"/>
       <c r="O47" t="n">
-        <v>12.45</v>
+        <v>13.65</v>
       </c>
       <c r="P47" t="n">
-        <v>281.9</v>
+        <v>309.04</v>
       </c>
       <c r="Q47" t="inlineStr"/>
       <c r="R47" t="n">
-        <v>24.9</v>
+        <v>27.3</v>
       </c>
       <c r="S47" t="n">
-        <v>563.8</v>
+        <v>618.09</v>
       </c>
       <c r="T47" t="inlineStr"/>
     </row>
@@ -7318,7 +7318,7 @@
         <v>33356.4</v>
       </c>
       <c r="E51" t="n">
-        <v>0.0672</v>
+        <v>0.06610000000000001</v>
       </c>
       <c r="F51" t="n">
         <v>0.0675</v>
@@ -7333,30 +7333,30 @@
         <v>2251.56</v>
       </c>
       <c r="J51" t="n">
-        <v>0.45</v>
+        <v>2.12</v>
       </c>
       <c r="K51" t="n">
-        <v>10.05</v>
+        <v>47.69</v>
       </c>
       <c r="L51" t="n">
-        <v>1.33</v>
+        <v>6.22</v>
       </c>
       <c r="M51" t="n">
-        <v>30.02</v>
+        <v>140.1</v>
       </c>
       <c r="N51" t="inlineStr"/>
       <c r="O51" t="n">
-        <v>2.22</v>
+        <v>10.37</v>
       </c>
       <c r="P51" t="n">
-        <v>50.03</v>
+        <v>233.49</v>
       </c>
       <c r="Q51" t="inlineStr"/>
       <c r="R51" t="n">
-        <v>4.44</v>
+        <v>20.74</v>
       </c>
       <c r="S51" t="n">
-        <v>100.07</v>
+        <v>466.99</v>
       </c>
       <c r="T51" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Update trade journals and leverage log (live bot activity)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/leverage_journal.xlsx
+++ b/leverage_journal.xlsx
@@ -459,10 +459,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-232.95</v>
+        <v>106.18</v>
       </c>
       <c r="C2" t="n">
-        <v>45.6</v>
+        <v>47.8</v>
       </c>
       <c r="D2" t="inlineStr"/>
     </row>
@@ -473,10 +473,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>888.99</v>
+        <v>2227.31</v>
       </c>
       <c r="C3" t="n">
-        <v>45.6</v>
+        <v>47.8</v>
       </c>
       <c r="D3" t="n">
         <v>1</v>
@@ -489,10 +489,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2482.98</v>
+        <v>4713.47</v>
       </c>
       <c r="C4" t="n">
-        <v>45.6</v>
+        <v>47.8</v>
       </c>
       <c r="D4" t="n">
         <v>1</v>
@@ -505,13 +505,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>18967.34</v>
+        <v>23502.04</v>
       </c>
       <c r="C5" t="n">
-        <v>45.6</v>
+        <v>47.8</v>
       </c>
       <c r="D5" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6">
@@ -521,10 +521,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3991.18</v>
+        <v>4937.17</v>
       </c>
       <c r="C6" t="n">
-        <v>52.9</v>
+        <v>50.7</v>
       </c>
       <c r="D6" t="inlineStr"/>
     </row>
@@ -535,10 +535,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>742.51</v>
+        <v>-274.85</v>
       </c>
       <c r="C7" t="n">
-        <v>52.9</v>
+        <v>50.7</v>
       </c>
       <c r="D7" t="n">
         <v>1</v>
@@ -551,10 +551,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2229.88</v>
+        <v>534.3200000000001</v>
       </c>
       <c r="C8" t="n">
-        <v>52.9</v>
+        <v>52.2</v>
       </c>
       <c r="D8" t="n">
         <v>5</v>
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>15984.55</v>
+        <v>12593.43</v>
       </c>
       <c r="C9" t="n">
-        <v>54.4</v>
+        <v>52.2</v>
       </c>
       <c r="D9" t="n">
         <v>16</v>
@@ -587,7 +587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T69"/>
+  <dimension ref="A1:T70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -713,7 +713,7 @@
         <v>1.589</v>
       </c>
       <c r="F2" t="n">
-        <v>1.426</v>
+        <v>1.434</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -725,36 +725,32 @@
         <v>20.04</v>
       </c>
       <c r="J2" t="n">
-        <v>-10.26</v>
+        <v>-9.75</v>
       </c>
       <c r="K2" t="n">
-        <v>-2.06</v>
+        <v>-1.95</v>
       </c>
       <c r="L2" t="n">
-        <v>-30.77</v>
+        <v>-29.26</v>
       </c>
       <c r="M2" t="n">
-        <v>-6.17</v>
+        <v>-5.86</v>
       </c>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="n">
-        <v>-51.29</v>
+        <v>-48.77</v>
       </c>
       <c r="P2" t="n">
-        <v>-10.28</v>
+        <v>-9.77</v>
       </c>
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="n">
-        <v>-100</v>
+        <v>-97.55</v>
       </c>
       <c r="S2" t="n">
-        <v>-20.04</v>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
+        <v>-19.55</v>
+      </c>
+      <c r="T2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -777,7 +773,7 @@
         <v>1.588</v>
       </c>
       <c r="F3" t="n">
-        <v>1.426</v>
+        <v>1.434</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -789,36 +785,32 @@
         <v>19.99</v>
       </c>
       <c r="J3" t="n">
-        <v>-10.2</v>
+        <v>-9.699999999999999</v>
       </c>
       <c r="K3" t="n">
-        <v>-2.04</v>
+        <v>-1.94</v>
       </c>
       <c r="L3" t="n">
-        <v>-30.6</v>
+        <v>-29.09</v>
       </c>
       <c r="M3" t="n">
-        <v>-6.12</v>
+        <v>-5.81</v>
       </c>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="n">
-        <v>-51.01</v>
+        <v>-48.49</v>
       </c>
       <c r="P3" t="n">
-        <v>-10.19</v>
+        <v>-9.69</v>
       </c>
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="n">
-        <v>-100</v>
+        <v>-96.98</v>
       </c>
       <c r="S3" t="n">
-        <v>-19.99</v>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
+        <v>-19.38</v>
+      </c>
+      <c r="T3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -841,7 +833,7 @@
         <v>1.59</v>
       </c>
       <c r="F4" t="n">
-        <v>1.426</v>
+        <v>1.434</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -853,36 +845,32 @@
         <v>20.01</v>
       </c>
       <c r="J4" t="n">
-        <v>-10.31</v>
+        <v>-9.81</v>
       </c>
       <c r="K4" t="n">
-        <v>-2.06</v>
+        <v>-1.96</v>
       </c>
       <c r="L4" t="n">
-        <v>-30.94</v>
+        <v>-29.43</v>
       </c>
       <c r="M4" t="n">
-        <v>-6.19</v>
+        <v>-5.89</v>
       </c>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="n">
-        <v>-51.57</v>
+        <v>-49.06</v>
       </c>
       <c r="P4" t="n">
-        <v>-10.32</v>
+        <v>-9.82</v>
       </c>
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="n">
-        <v>-100</v>
+        <v>-98.11</v>
       </c>
       <c r="S4" t="n">
-        <v>-20.01</v>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
+        <v>-19.63</v>
+      </c>
+      <c r="T4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -969,7 +957,7 @@
         <v>0.000529</v>
       </c>
       <c r="F6" t="n">
-        <v>0.00051</v>
+        <v>0.000496</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -981,27 +969,27 @@
         <v>0.02</v>
       </c>
       <c r="J6" t="n">
-        <v>-3.59</v>
+        <v>-6.24</v>
       </c>
       <c r="K6" t="n">
         <v>-0</v>
       </c>
       <c r="L6" t="n">
-        <v>-10.78</v>
+        <v>-18.71</v>
       </c>
       <c r="M6" t="n">
         <v>-0</v>
       </c>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="n">
-        <v>-17.96</v>
+        <v>-31.19</v>
       </c>
       <c r="P6" t="n">
-        <v>-0</v>
+        <v>-0.01</v>
       </c>
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="n">
-        <v>-35.92</v>
+        <v>-62.38</v>
       </c>
       <c r="S6" t="n">
         <v>-0.01</v>
@@ -2085,7 +2073,7 @@
         <v>2.68</v>
       </c>
       <c r="F23" t="n">
-        <v>2.432</v>
+        <v>2.258</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -2097,32 +2085,36 @@
         <v>5.87</v>
       </c>
       <c r="J23" t="n">
-        <v>-9.25</v>
+        <v>-15.75</v>
       </c>
       <c r="K23" t="n">
-        <v>-0.54</v>
+        <v>-0.92</v>
       </c>
       <c r="L23" t="n">
-        <v>-27.76</v>
+        <v>-47.24</v>
       </c>
       <c r="M23" t="n">
-        <v>-1.63</v>
+        <v>-2.77</v>
       </c>
       <c r="N23" t="inlineStr"/>
       <c r="O23" t="n">
-        <v>-46.27</v>
+        <v>-78.73</v>
       </c>
       <c r="P23" t="n">
-        <v>-2.72</v>
+        <v>-4.62</v>
       </c>
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="n">
-        <v>-92.54000000000001</v>
+        <v>-100</v>
       </c>
       <c r="S23" t="n">
-        <v>-5.43</v>
-      </c>
-      <c r="T23" t="inlineStr"/>
+        <v>-5.87</v>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -3701,7 +3693,7 @@
         <v>0.1769</v>
       </c>
       <c r="F48" t="n">
-        <v>0.0556</v>
+        <v>0.043</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -3713,10 +3705,10 @@
         <v>1502.06</v>
       </c>
       <c r="J48" t="n">
-        <v>-68.56999999999999</v>
+        <v>-75.69</v>
       </c>
       <c r="K48" t="n">
-        <v>-1029.96</v>
+        <v>-1136.94</v>
       </c>
       <c r="L48" t="n">
         <v>-100</v>
@@ -4285,7 +4277,7 @@
         <v>0.01825474902120262</v>
       </c>
       <c r="F57" t="n">
-        <v>0.01817</v>
+        <v>0.0191</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
@@ -4297,30 +4289,30 @@
         <v>2289.31</v>
       </c>
       <c r="J57" t="n">
-        <v>-0.46</v>
+        <v>4.63</v>
       </c>
       <c r="K57" t="n">
-        <v>-10.63</v>
+        <v>106</v>
       </c>
       <c r="L57" t="n">
-        <v>-1.39</v>
+        <v>13.89</v>
       </c>
       <c r="M57" t="n">
-        <v>-31.88</v>
+        <v>318.01</v>
       </c>
       <c r="N57" t="inlineStr"/>
       <c r="O57" t="n">
-        <v>-2.32</v>
+        <v>23.15</v>
       </c>
       <c r="P57" t="n">
-        <v>-53.14</v>
+        <v>530.01</v>
       </c>
       <c r="Q57" t="inlineStr"/>
       <c r="R57" t="n">
-        <v>-4.64</v>
+        <v>46.3</v>
       </c>
       <c r="S57" t="n">
-        <v>-106.28</v>
+        <v>1060.02</v>
       </c>
       <c r="T57" t="inlineStr"/>
     </row>
@@ -4463,52 +4455,56 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>CLOSED</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>9356</v>
+        <v>9355</v>
       </c>
       <c r="E60" t="n">
         <v>0.07548835965087614</v>
       </c>
       <c r="F60" t="n">
-        <v>0.06426999999999999</v>
+        <v>0.06350149652592196</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
           <t>2026-07-30 17:18</t>
         </is>
       </c>
-      <c r="H60" t="inlineStr"/>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>2026-08-03 01:06</t>
+        </is>
+      </c>
       <c r="I60" t="n">
-        <v>706.27</v>
+        <v>706.1900000000001</v>
       </c>
       <c r="J60" t="n">
-        <v>-14.86</v>
+        <v>-15.88</v>
       </c>
       <c r="K60" t="n">
-        <v>-104.96</v>
+        <v>-112.14</v>
       </c>
       <c r="L60" t="n">
-        <v>-44.58</v>
+        <v>-47.64</v>
       </c>
       <c r="M60" t="n">
-        <v>-314.88</v>
+        <v>-336.41</v>
       </c>
       <c r="N60" t="inlineStr"/>
       <c r="O60" t="n">
-        <v>-74.31</v>
+        <v>-79.40000000000001</v>
       </c>
       <c r="P60" t="n">
-        <v>-524.79</v>
+        <v>-560.6900000000001</v>
       </c>
       <c r="Q60" t="inlineStr"/>
       <c r="R60" t="n">
         <v>-100</v>
       </c>
       <c r="S60" t="n">
-        <v>-706.27</v>
+        <v>-706.1900000000001</v>
       </c>
       <c r="T60" t="inlineStr">
         <is>
@@ -4522,7 +4518,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>PEOPLE</t>
+          <t>ESP</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -4531,50 +4527,54 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>653866.1</v>
+        <v>1</v>
       </c>
       <c r="E61" t="n">
-        <v>0.006940588409461815</v>
+        <v>0.07548835965087614</v>
       </c>
       <c r="F61" t="n">
-        <v>0.00653</v>
+        <v>0.06585000000000001</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>2026-07-30 17:47</t>
+          <t>2026-07-30 17:18</t>
         </is>
       </c>
       <c r="H61" t="inlineStr"/>
       <c r="I61" t="n">
-        <v>4538.22</v>
+        <v>0.08</v>
       </c>
       <c r="J61" t="n">
-        <v>-5.92</v>
+        <v>-12.77</v>
       </c>
       <c r="K61" t="n">
-        <v>-268.47</v>
+        <v>-0.01</v>
       </c>
       <c r="L61" t="n">
-        <v>-17.75</v>
+        <v>-38.3</v>
       </c>
       <c r="M61" t="n">
-        <v>-805.41</v>
+        <v>-0.03</v>
       </c>
       <c r="N61" t="inlineStr"/>
       <c r="O61" t="n">
-        <v>-29.58</v>
+        <v>-63.84</v>
       </c>
       <c r="P61" t="n">
-        <v>-1342.35</v>
+        <v>-0.05</v>
       </c>
       <c r="Q61" t="inlineStr"/>
       <c r="R61" t="n">
-        <v>-59.16</v>
+        <v>-100</v>
       </c>
       <c r="S61" t="n">
-        <v>-2684.7</v>
-      </c>
-      <c r="T61" t="inlineStr"/>
+        <v>-0.08</v>
+      </c>
+      <c r="T61" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -4582,61 +4582,57 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>ROBO</t>
+          <t>PEOPLE</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>CLOSED</t>
+          <t>OPEN</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>220379</v>
+        <v>653866.1</v>
       </c>
       <c r="E62" t="n">
-        <v>0.0135</v>
+        <v>0.006940588409461815</v>
       </c>
       <c r="F62" t="n">
-        <v>0.01228</v>
+        <v>0.00712</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>2026-07-31 08:27</t>
-        </is>
-      </c>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>2026-07-31 16:30</t>
-        </is>
-      </c>
+          <t>2026-07-30 17:47</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr"/>
       <c r="I62" t="n">
-        <v>2975.12</v>
+        <v>4538.22</v>
       </c>
       <c r="J62" t="n">
-        <v>-9.039999999999999</v>
+        <v>2.58</v>
       </c>
       <c r="K62" t="n">
-        <v>-268.86</v>
+        <v>117.31</v>
       </c>
       <c r="L62" t="n">
-        <v>-27.11</v>
+        <v>7.75</v>
       </c>
       <c r="M62" t="n">
-        <v>-806.59</v>
+        <v>351.93</v>
       </c>
       <c r="N62" t="inlineStr"/>
       <c r="O62" t="n">
-        <v>-45.19</v>
+        <v>12.92</v>
       </c>
       <c r="P62" t="n">
-        <v>-1344.31</v>
+        <v>586.5599999999999</v>
       </c>
       <c r="Q62" t="inlineStr"/>
       <c r="R62" t="n">
-        <v>-90.37</v>
+        <v>25.85</v>
       </c>
       <c r="S62" t="n">
-        <v>-2688.62</v>
+        <v>1173.11</v>
       </c>
       <c r="T62" t="inlineStr"/>
     </row>
@@ -4655,7 +4651,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>110190</v>
+        <v>220379</v>
       </c>
       <c r="E63" t="n">
         <v>0.0135</v>
@@ -4674,33 +4670,33 @@
         </is>
       </c>
       <c r="I63" t="n">
-        <v>1487.57</v>
+        <v>2975.12</v>
       </c>
       <c r="J63" t="n">
         <v>-9.039999999999999</v>
       </c>
       <c r="K63" t="n">
-        <v>-134.43</v>
+        <v>-268.86</v>
       </c>
       <c r="L63" t="n">
         <v>-27.11</v>
       </c>
       <c r="M63" t="n">
-        <v>-403.3</v>
+        <v>-806.59</v>
       </c>
       <c r="N63" t="inlineStr"/>
       <c r="O63" t="n">
         <v>-45.19</v>
       </c>
       <c r="P63" t="n">
-        <v>-672.16</v>
+        <v>-1344.31</v>
       </c>
       <c r="Q63" t="inlineStr"/>
       <c r="R63" t="n">
         <v>-90.37</v>
       </c>
       <c r="S63" t="n">
-        <v>-1344.32</v>
+        <v>-2688.62</v>
       </c>
       <c r="T63" t="inlineStr"/>
     </row>
@@ -4710,57 +4706,61 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>CFX</t>
+          <t>ROBO</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>CLOSED</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>106828</v>
+        <v>110190</v>
       </c>
       <c r="E64" t="n">
-        <v>0.04149347287228067</v>
+        <v>0.0135</v>
       </c>
       <c r="F64" t="n">
-        <v>0.04294</v>
+        <v>0.01228</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>2026-07-31 13:00</t>
-        </is>
-      </c>
-      <c r="H64" t="inlineStr"/>
+          <t>2026-07-31 08:27</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>2026-07-31 16:30</t>
+        </is>
+      </c>
       <c r="I64" t="n">
-        <v>4432.66</v>
+        <v>1487.57</v>
       </c>
       <c r="J64" t="n">
-        <v>3.49</v>
+        <v>-9.039999999999999</v>
       </c>
       <c r="K64" t="n">
-        <v>154.53</v>
+        <v>-134.43</v>
       </c>
       <c r="L64" t="n">
-        <v>10.46</v>
+        <v>-27.11</v>
       </c>
       <c r="M64" t="n">
-        <v>463.59</v>
+        <v>-403.3</v>
       </c>
       <c r="N64" t="inlineStr"/>
       <c r="O64" t="n">
-        <v>17.43</v>
+        <v>-45.19</v>
       </c>
       <c r="P64" t="n">
-        <v>772.65</v>
+        <v>-672.16</v>
       </c>
       <c r="Q64" t="inlineStr"/>
       <c r="R64" t="n">
-        <v>34.86</v>
+        <v>-90.37</v>
       </c>
       <c r="S64" t="n">
-        <v>1545.3</v>
+        <v>-1344.32</v>
       </c>
       <c r="T64" t="inlineStr"/>
     </row>
@@ -4770,7 +4770,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>GMT</t>
+          <t>CFX</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -4779,48 +4779,48 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>325667.9</v>
+        <v>106828</v>
       </c>
       <c r="E65" t="n">
-        <v>0.00676</v>
+        <v>0.04149347287228067</v>
       </c>
       <c r="F65" t="n">
-        <v>0.00663</v>
+        <v>0.04085</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>2026-07-31 13:55</t>
+          <t>2026-07-31 13:00</t>
         </is>
       </c>
       <c r="H65" t="inlineStr"/>
       <c r="I65" t="n">
-        <v>2201.52</v>
+        <v>4432.66</v>
       </c>
       <c r="J65" t="n">
-        <v>-1.92</v>
+        <v>-1.55</v>
       </c>
       <c r="K65" t="n">
-        <v>-42.34</v>
+        <v>-68.73999999999999</v>
       </c>
       <c r="L65" t="n">
-        <v>-5.77</v>
+        <v>-4.65</v>
       </c>
       <c r="M65" t="n">
-        <v>-127.01</v>
+        <v>-206.22</v>
       </c>
       <c r="N65" t="inlineStr"/>
       <c r="O65" t="n">
-        <v>-9.619999999999999</v>
+        <v>-7.75</v>
       </c>
       <c r="P65" t="n">
-        <v>-211.68</v>
+        <v>-343.7</v>
       </c>
       <c r="Q65" t="inlineStr"/>
       <c r="R65" t="n">
-        <v>-19.23</v>
+        <v>-15.51</v>
       </c>
       <c r="S65" t="n">
-        <v>-423.37</v>
+        <v>-687.41</v>
       </c>
       <c r="T65" t="inlineStr"/>
     </row>
@@ -4830,7 +4830,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>SAGA</t>
+          <t>GMT</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -4839,48 +4839,48 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>339939.6</v>
+        <v>325667.9</v>
       </c>
       <c r="E66" t="n">
-        <v>0.0126</v>
+        <v>0.00676</v>
       </c>
       <c r="F66" t="n">
-        <v>0.01236</v>
+        <v>0.00657</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>2026-07-31 17:04</t>
+          <t>2026-07-31 13:55</t>
         </is>
       </c>
       <c r="H66" t="inlineStr"/>
       <c r="I66" t="n">
-        <v>4283.24</v>
+        <v>2201.52</v>
       </c>
       <c r="J66" t="n">
-        <v>-1.9</v>
+        <v>-2.81</v>
       </c>
       <c r="K66" t="n">
-        <v>-81.59</v>
+        <v>-61.88</v>
       </c>
       <c r="L66" t="n">
-        <v>-5.71</v>
+        <v>-8.43</v>
       </c>
       <c r="M66" t="n">
-        <v>-244.76</v>
+        <v>-185.63</v>
       </c>
       <c r="N66" t="inlineStr"/>
       <c r="O66" t="n">
-        <v>-9.52</v>
+        <v>-14.05</v>
       </c>
       <c r="P66" t="n">
-        <v>-407.93</v>
+        <v>-309.38</v>
       </c>
       <c r="Q66" t="inlineStr"/>
       <c r="R66" t="n">
-        <v>-19.05</v>
+        <v>-28.11</v>
       </c>
       <c r="S66" t="n">
-        <v>-815.86</v>
+        <v>-618.77</v>
       </c>
       <c r="T66" t="inlineStr"/>
     </row>
@@ -4890,61 +4890,57 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>FLOW</t>
+          <t>SAGA</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>CLOSED</t>
+          <t>OPEN</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>97950.02</v>
+        <v>339939.6</v>
       </c>
       <c r="E67" t="n">
-        <v>0.02804405102724839</v>
+        <v>0.0126</v>
       </c>
       <c r="F67" t="n">
-        <v>0.03081</v>
+        <v>0.01293</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>2026-07-31 17:13</t>
-        </is>
-      </c>
-      <c r="H67" t="inlineStr">
-        <is>
-          <t>2026-07-31 23:28</t>
-        </is>
-      </c>
+          <t>2026-07-31 17:04</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr"/>
       <c r="I67" t="n">
-        <v>2746.92</v>
+        <v>4283.24</v>
       </c>
       <c r="J67" t="n">
-        <v>9.859999999999999</v>
+        <v>2.62</v>
       </c>
       <c r="K67" t="n">
-        <v>270.92</v>
+        <v>112.18</v>
       </c>
       <c r="L67" t="n">
-        <v>29.59</v>
+        <v>7.86</v>
       </c>
       <c r="M67" t="n">
-        <v>812.77</v>
+        <v>336.54</v>
       </c>
       <c r="N67" t="inlineStr"/>
       <c r="O67" t="n">
-        <v>49.31</v>
+        <v>13.1</v>
       </c>
       <c r="P67" t="n">
-        <v>1354.62</v>
+        <v>560.9</v>
       </c>
       <c r="Q67" t="inlineStr"/>
       <c r="R67" t="n">
-        <v>98.63</v>
+        <v>26.19</v>
       </c>
       <c r="S67" t="n">
-        <v>2709.25</v>
+        <v>1121.8</v>
       </c>
       <c r="T67" t="inlineStr"/>
     </row>
@@ -4954,7 +4950,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>TLM</t>
+          <t>FLOW</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -4963,58 +4959,54 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>765466</v>
+        <v>97950.02</v>
       </c>
       <c r="E68" t="n">
-        <v>0.001873560456366487</v>
+        <v>0.02804405102724839</v>
       </c>
       <c r="F68" t="n">
-        <v>0.001648650814013947</v>
+        <v>0.03081</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>2026-08-01 07:57</t>
+          <t>2026-07-31 17:13</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>2026-08-01 10:31</t>
+          <t>2026-07-31 23:28</t>
         </is>
       </c>
       <c r="I68" t="n">
-        <v>1434.15</v>
+        <v>2746.92</v>
       </c>
       <c r="J68" t="n">
-        <v>-12</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="K68" t="n">
-        <v>-172.16</v>
+        <v>270.92</v>
       </c>
       <c r="L68" t="n">
-        <v>-36.01</v>
+        <v>29.59</v>
       </c>
       <c r="M68" t="n">
-        <v>-516.48</v>
+        <v>812.77</v>
       </c>
       <c r="N68" t="inlineStr"/>
       <c r="O68" t="n">
-        <v>-60.02</v>
+        <v>49.31</v>
       </c>
       <c r="P68" t="n">
-        <v>-860.8</v>
+        <v>1354.62</v>
       </c>
       <c r="Q68" t="inlineStr"/>
       <c r="R68" t="n">
-        <v>-100</v>
+        <v>98.63</v>
       </c>
       <c r="S68" t="n">
-        <v>-1434.15</v>
-      </c>
-      <c r="T68" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
+        <v>2709.25</v>
+      </c>
+      <c r="T68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -5031,13 +5023,13 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>382734</v>
+        <v>765466</v>
       </c>
       <c r="E69" t="n">
         <v>0.001873560456366487</v>
       </c>
       <c r="F69" t="n">
-        <v>0.001648</v>
+        <v>0.001648650814013947</v>
       </c>
       <c r="G69" t="inlineStr">
         <is>
@@ -5050,35 +5042,103 @@
         </is>
       </c>
       <c r="I69" t="n">
-        <v>717.08</v>
+        <v>1434.15</v>
       </c>
       <c r="J69" t="n">
-        <v>-12.04</v>
+        <v>-12</v>
       </c>
       <c r="K69" t="n">
-        <v>-86.33</v>
+        <v>-172.16</v>
       </c>
       <c r="L69" t="n">
-        <v>-36.12</v>
+        <v>-36.01</v>
       </c>
       <c r="M69" t="n">
-        <v>-258.99</v>
+        <v>-516.48</v>
       </c>
       <c r="N69" t="inlineStr"/>
       <c r="O69" t="n">
-        <v>-60.2</v>
+        <v>-60.02</v>
       </c>
       <c r="P69" t="n">
-        <v>-431.65</v>
+        <v>-860.8</v>
       </c>
       <c r="Q69" t="inlineStr"/>
       <c r="R69" t="n">
         <v>-100</v>
       </c>
       <c r="S69" t="n">
+        <v>-1434.15</v>
+      </c>
+      <c r="T69" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>TLM</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>382734</v>
+      </c>
+      <c r="E70" t="n">
+        <v>0.001873560456366487</v>
+      </c>
+      <c r="F70" t="n">
+        <v>0.001648</v>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>2026-08-01 07:57</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>2026-08-01 10:31</t>
+        </is>
+      </c>
+      <c r="I70" t="n">
+        <v>717.08</v>
+      </c>
+      <c r="J70" t="n">
+        <v>-12.04</v>
+      </c>
+      <c r="K70" t="n">
+        <v>-86.33</v>
+      </c>
+      <c r="L70" t="n">
+        <v>-36.12</v>
+      </c>
+      <c r="M70" t="n">
+        <v>-258.99</v>
+      </c>
+      <c r="N70" t="inlineStr"/>
+      <c r="O70" t="n">
+        <v>-60.2</v>
+      </c>
+      <c r="P70" t="n">
+        <v>-431.65</v>
+      </c>
+      <c r="Q70" t="inlineStr"/>
+      <c r="R70" t="n">
+        <v>-100</v>
+      </c>
+      <c r="S70" t="n">
         <v>-717.08</v>
       </c>
-      <c r="T69" t="inlineStr">
+      <c r="T70" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -5095,7 +5155,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T69"/>
+  <dimension ref="A1:T70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5218,7 +5278,7 @@
         <v>12.61</v>
       </c>
       <c r="E2" t="n">
-        <v>1.426</v>
+        <v>1.434</v>
       </c>
       <c r="F2" t="n">
         <v>1.589</v>
@@ -5233,30 +5293,30 @@
         <v>20.04</v>
       </c>
       <c r="J2" t="n">
-        <v>11.43</v>
+        <v>10.81</v>
       </c>
       <c r="K2" t="n">
-        <v>2.29</v>
+        <v>2.17</v>
       </c>
       <c r="L2" t="n">
-        <v>30.77</v>
+        <v>29.26</v>
       </c>
       <c r="M2" t="n">
-        <v>6.17</v>
+        <v>5.86</v>
       </c>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="n">
-        <v>51.29</v>
+        <v>48.77</v>
       </c>
       <c r="P2" t="n">
-        <v>10.28</v>
+        <v>9.77</v>
       </c>
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="n">
-        <v>102.58</v>
+        <v>97.55</v>
       </c>
       <c r="S2" t="n">
-        <v>20.55</v>
+        <v>19.55</v>
       </c>
       <c r="T2" t="inlineStr"/>
     </row>
@@ -5278,7 +5338,7 @@
         <v>12.586</v>
       </c>
       <c r="E3" t="n">
-        <v>1.426</v>
+        <v>1.434</v>
       </c>
       <c r="F3" t="n">
         <v>1.588</v>
@@ -5293,30 +5353,30 @@
         <v>19.99</v>
       </c>
       <c r="J3" t="n">
-        <v>11.36</v>
+        <v>10.74</v>
       </c>
       <c r="K3" t="n">
-        <v>2.27</v>
+        <v>2.15</v>
       </c>
       <c r="L3" t="n">
-        <v>30.6</v>
+        <v>29.09</v>
       </c>
       <c r="M3" t="n">
-        <v>6.12</v>
+        <v>5.81</v>
       </c>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="n">
-        <v>51.01</v>
+        <v>48.49</v>
       </c>
       <c r="P3" t="n">
-        <v>10.19</v>
+        <v>9.69</v>
       </c>
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="n">
-        <v>102.02</v>
+        <v>96.98</v>
       </c>
       <c r="S3" t="n">
-        <v>20.39</v>
+        <v>19.38</v>
       </c>
       <c r="T3" t="inlineStr"/>
     </row>
@@ -5338,7 +5398,7 @@
         <v>12.586</v>
       </c>
       <c r="E4" t="n">
-        <v>1.426</v>
+        <v>1.434</v>
       </c>
       <c r="F4" t="n">
         <v>1.59</v>
@@ -5353,30 +5413,30 @@
         <v>20.01</v>
       </c>
       <c r="J4" t="n">
-        <v>11.5</v>
+        <v>10.88</v>
       </c>
       <c r="K4" t="n">
-        <v>2.3</v>
+        <v>2.18</v>
       </c>
       <c r="L4" t="n">
-        <v>30.94</v>
+        <v>29.43</v>
       </c>
       <c r="M4" t="n">
-        <v>6.19</v>
+        <v>5.89</v>
       </c>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="n">
-        <v>51.57</v>
+        <v>49.06</v>
       </c>
       <c r="P4" t="n">
-        <v>10.32</v>
+        <v>9.82</v>
       </c>
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="n">
-        <v>103.14</v>
+        <v>98.11</v>
       </c>
       <c r="S4" t="n">
-        <v>20.64</v>
+        <v>19.63</v>
       </c>
       <c r="T4" t="inlineStr"/>
     </row>
@@ -5462,7 +5522,7 @@
         <v>38</v>
       </c>
       <c r="E6" t="n">
-        <v>0.00051</v>
+        <v>0.000496</v>
       </c>
       <c r="F6" t="n">
         <v>0.000529</v>
@@ -5477,27 +5537,27 @@
         <v>0.02</v>
       </c>
       <c r="J6" t="n">
-        <v>3.73</v>
+        <v>6.65</v>
       </c>
       <c r="K6" t="n">
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>10.78</v>
+        <v>18.71</v>
       </c>
       <c r="M6" t="n">
         <v>0</v>
       </c>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="n">
-        <v>17.96</v>
+        <v>31.19</v>
       </c>
       <c r="P6" t="n">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="n">
-        <v>35.92</v>
+        <v>62.38</v>
       </c>
       <c r="S6" t="n">
         <v>0.01</v>
@@ -6574,7 +6634,7 @@
         <v>2.19</v>
       </c>
       <c r="E23" t="n">
-        <v>2.432</v>
+        <v>2.258</v>
       </c>
       <c r="F23" t="n">
         <v>2.68</v>
@@ -6589,30 +6649,30 @@
         <v>5.87</v>
       </c>
       <c r="J23" t="n">
-        <v>10.2</v>
+        <v>18.69</v>
       </c>
       <c r="K23" t="n">
-        <v>0.6</v>
+        <v>1.1</v>
       </c>
       <c r="L23" t="n">
-        <v>27.76</v>
+        <v>47.24</v>
       </c>
       <c r="M23" t="n">
-        <v>1.63</v>
+        <v>2.77</v>
       </c>
       <c r="N23" t="inlineStr"/>
       <c r="O23" t="n">
-        <v>46.27</v>
+        <v>78.73</v>
       </c>
       <c r="P23" t="n">
-        <v>2.72</v>
+        <v>4.62</v>
       </c>
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="n">
-        <v>92.54000000000001</v>
+        <v>157.46</v>
       </c>
       <c r="S23" t="n">
-        <v>5.43</v>
+        <v>9.24</v>
       </c>
       <c r="T23" t="inlineStr"/>
     </row>
@@ -8198,7 +8258,7 @@
         <v>8491</v>
       </c>
       <c r="E48" t="n">
-        <v>0.0556</v>
+        <v>0.043</v>
       </c>
       <c r="F48" t="n">
         <v>0.1769</v>
@@ -8213,30 +8273,30 @@
         <v>1502.06</v>
       </c>
       <c r="J48" t="n">
-        <v>218.17</v>
+        <v>311.4</v>
       </c>
       <c r="K48" t="n">
-        <v>3276.97</v>
+        <v>4677.34</v>
       </c>
       <c r="L48" t="n">
-        <v>205.71</v>
+        <v>227.08</v>
       </c>
       <c r="M48" t="n">
-        <v>3089.87</v>
+        <v>3410.83</v>
       </c>
       <c r="N48" t="inlineStr"/>
       <c r="O48" t="n">
-        <v>342.85</v>
+        <v>378.46</v>
       </c>
       <c r="P48" t="n">
-        <v>5149.79</v>
+        <v>5684.72</v>
       </c>
       <c r="Q48" t="inlineStr"/>
       <c r="R48" t="n">
-        <v>685.7</v>
+        <v>756.92</v>
       </c>
       <c r="S48" t="n">
-        <v>10299.58</v>
+        <v>11369.45</v>
       </c>
       <c r="T48" t="inlineStr"/>
     </row>
@@ -8782,7 +8842,7 @@
         <v>125409</v>
       </c>
       <c r="E57" t="n">
-        <v>0.01817</v>
+        <v>0.0191</v>
       </c>
       <c r="F57" t="n">
         <v>0.01825474902120262</v>
@@ -8797,30 +8857,30 @@
         <v>2289.31</v>
       </c>
       <c r="J57" t="n">
-        <v>0.47</v>
+        <v>-4.43</v>
       </c>
       <c r="K57" t="n">
-        <v>10.68</v>
+        <v>-101.31</v>
       </c>
       <c r="L57" t="n">
-        <v>1.39</v>
+        <v>-13.89</v>
       </c>
       <c r="M57" t="n">
-        <v>31.88</v>
+        <v>-318.01</v>
       </c>
       <c r="N57" t="inlineStr"/>
       <c r="O57" t="n">
-        <v>2.32</v>
+        <v>-23.15</v>
       </c>
       <c r="P57" t="n">
-        <v>53.14</v>
+        <v>-530.01</v>
       </c>
       <c r="Q57" t="inlineStr"/>
       <c r="R57" t="n">
-        <v>4.64</v>
+        <v>-46.3</v>
       </c>
       <c r="S57" t="n">
-        <v>106.28</v>
+        <v>-1060.02</v>
       </c>
       <c r="T57" t="inlineStr"/>
     </row>
@@ -8983,14 +9043,14 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>CLOSED</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>9356</v>
+        <v>9355</v>
       </c>
       <c r="E60" t="n">
-        <v>0.06426999999999999</v>
+        <v>0.06350149652592196</v>
       </c>
       <c r="F60" t="n">
         <v>0.07548835965087614</v>
@@ -9000,35 +9060,39 @@
           <t>2026-07-30 17:18</t>
         </is>
       </c>
-      <c r="H60" t="inlineStr"/>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>2026-08-03 01:06</t>
+        </is>
+      </c>
       <c r="I60" t="n">
-        <v>706.27</v>
+        <v>706.1900000000001</v>
       </c>
       <c r="J60" t="n">
-        <v>17.46</v>
+        <v>18.88</v>
       </c>
       <c r="K60" t="n">
-        <v>123.28</v>
+        <v>133.3</v>
       </c>
       <c r="L60" t="n">
-        <v>44.58</v>
+        <v>47.64</v>
       </c>
       <c r="M60" t="n">
-        <v>314.88</v>
+        <v>336.41</v>
       </c>
       <c r="N60" t="inlineStr"/>
       <c r="O60" t="n">
-        <v>74.31</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="P60" t="n">
-        <v>524.79</v>
+        <v>560.6900000000001</v>
       </c>
       <c r="Q60" t="inlineStr"/>
       <c r="R60" t="n">
-        <v>148.61</v>
+        <v>158.79</v>
       </c>
       <c r="S60" t="n">
-        <v>1049.59</v>
+        <v>1121.37</v>
       </c>
       <c r="T60" t="inlineStr"/>
     </row>
@@ -9038,7 +9102,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>PEOPLE</t>
+          <t>ESP</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -9047,48 +9111,48 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>653866.1</v>
+        <v>1</v>
       </c>
       <c r="E61" t="n">
-        <v>0.00653</v>
+        <v>0.06585000000000001</v>
       </c>
       <c r="F61" t="n">
-        <v>0.006940588409461815</v>
+        <v>0.07548835965087614</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>2026-07-30 17:47</t>
+          <t>2026-07-30 17:18</t>
         </is>
       </c>
       <c r="H61" t="inlineStr"/>
       <c r="I61" t="n">
-        <v>4538.22</v>
+        <v>0.08</v>
       </c>
       <c r="J61" t="n">
-        <v>6.29</v>
+        <v>14.64</v>
       </c>
       <c r="K61" t="n">
-        <v>285.35</v>
+        <v>0.01</v>
       </c>
       <c r="L61" t="n">
-        <v>17.75</v>
+        <v>38.3</v>
       </c>
       <c r="M61" t="n">
-        <v>805.41</v>
+        <v>0.03</v>
       </c>
       <c r="N61" t="inlineStr"/>
       <c r="O61" t="n">
-        <v>29.58</v>
+        <v>63.84</v>
       </c>
       <c r="P61" t="n">
-        <v>1342.35</v>
+        <v>0.05</v>
       </c>
       <c r="Q61" t="inlineStr"/>
       <c r="R61" t="n">
-        <v>59.16</v>
+        <v>127.68</v>
       </c>
       <c r="S61" t="n">
-        <v>2684.7</v>
+        <v>0.1</v>
       </c>
       <c r="T61" t="inlineStr"/>
     </row>
@@ -9098,61 +9162,57 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>ROBO</t>
+          <t>PEOPLE</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>CLOSED</t>
+          <t>OPEN</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>220379</v>
+        <v>653866.1</v>
       </c>
       <c r="E62" t="n">
-        <v>0.01228</v>
+        <v>0.00712</v>
       </c>
       <c r="F62" t="n">
-        <v>0.0135</v>
+        <v>0.006940588409461815</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>2026-07-31 08:27</t>
-        </is>
-      </c>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>2026-07-31 16:30</t>
-        </is>
-      </c>
+          <t>2026-07-30 17:47</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr"/>
       <c r="I62" t="n">
-        <v>2975.12</v>
+        <v>4538.22</v>
       </c>
       <c r="J62" t="n">
-        <v>9.93</v>
+        <v>-2.52</v>
       </c>
       <c r="K62" t="n">
-        <v>295.57</v>
+        <v>-114.36</v>
       </c>
       <c r="L62" t="n">
-        <v>27.11</v>
+        <v>-7.75</v>
       </c>
       <c r="M62" t="n">
-        <v>806.59</v>
+        <v>-351.93</v>
       </c>
       <c r="N62" t="inlineStr"/>
       <c r="O62" t="n">
-        <v>45.19</v>
+        <v>-12.92</v>
       </c>
       <c r="P62" t="n">
-        <v>1344.31</v>
+        <v>-586.5599999999999</v>
       </c>
       <c r="Q62" t="inlineStr"/>
       <c r="R62" t="n">
-        <v>90.37</v>
+        <v>-25.85</v>
       </c>
       <c r="S62" t="n">
-        <v>2688.62</v>
+        <v>-1173.11</v>
       </c>
       <c r="T62" t="inlineStr"/>
     </row>
@@ -9171,7 +9231,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>110190</v>
+        <v>220379</v>
       </c>
       <c r="E63" t="n">
         <v>0.01228</v>
@@ -9190,33 +9250,33 @@
         </is>
       </c>
       <c r="I63" t="n">
-        <v>1487.57</v>
+        <v>2975.12</v>
       </c>
       <c r="J63" t="n">
         <v>9.93</v>
       </c>
       <c r="K63" t="n">
-        <v>147.79</v>
+        <v>295.57</v>
       </c>
       <c r="L63" t="n">
         <v>27.11</v>
       </c>
       <c r="M63" t="n">
-        <v>403.3</v>
+        <v>806.59</v>
       </c>
       <c r="N63" t="inlineStr"/>
       <c r="O63" t="n">
         <v>45.19</v>
       </c>
       <c r="P63" t="n">
-        <v>672.16</v>
+        <v>1344.31</v>
       </c>
       <c r="Q63" t="inlineStr"/>
       <c r="R63" t="n">
         <v>90.37</v>
       </c>
       <c r="S63" t="n">
-        <v>1344.32</v>
+        <v>2688.62</v>
       </c>
       <c r="T63" t="inlineStr"/>
     </row>
@@ -9226,57 +9286,61 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>CFX</t>
+          <t>ROBO</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>CLOSED</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>106828</v>
+        <v>110190</v>
       </c>
       <c r="E64" t="n">
-        <v>0.04294</v>
+        <v>0.01228</v>
       </c>
       <c r="F64" t="n">
-        <v>0.04149347287228067</v>
+        <v>0.0135</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>2026-07-31 13:00</t>
-        </is>
-      </c>
-      <c r="H64" t="inlineStr"/>
+          <t>2026-07-31 08:27</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>2026-07-31 16:30</t>
+        </is>
+      </c>
       <c r="I64" t="n">
-        <v>4432.66</v>
+        <v>1487.57</v>
       </c>
       <c r="J64" t="n">
-        <v>-3.37</v>
+        <v>9.93</v>
       </c>
       <c r="K64" t="n">
-        <v>-149.32</v>
+        <v>147.79</v>
       </c>
       <c r="L64" t="n">
-        <v>-10.46</v>
+        <v>27.11</v>
       </c>
       <c r="M64" t="n">
-        <v>-463.59</v>
+        <v>403.3</v>
       </c>
       <c r="N64" t="inlineStr"/>
       <c r="O64" t="n">
-        <v>-17.43</v>
+        <v>45.19</v>
       </c>
       <c r="P64" t="n">
-        <v>-772.65</v>
+        <v>672.16</v>
       </c>
       <c r="Q64" t="inlineStr"/>
       <c r="R64" t="n">
-        <v>-34.86</v>
+        <v>90.37</v>
       </c>
       <c r="S64" t="n">
-        <v>-1545.3</v>
+        <v>1344.32</v>
       </c>
       <c r="T64" t="inlineStr"/>
     </row>
@@ -9286,7 +9350,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>GMT</t>
+          <t>CFX</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -9295,48 +9359,48 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>325667.9</v>
+        <v>106828</v>
       </c>
       <c r="E65" t="n">
-        <v>0.00663</v>
+        <v>0.04085</v>
       </c>
       <c r="F65" t="n">
-        <v>0.00676</v>
+        <v>0.04149347287228067</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>2026-07-31 13:55</t>
+          <t>2026-07-31 13:00</t>
         </is>
       </c>
       <c r="H65" t="inlineStr"/>
       <c r="I65" t="n">
-        <v>2201.52</v>
+        <v>4432.66</v>
       </c>
       <c r="J65" t="n">
-        <v>1.96</v>
+        <v>1.58</v>
       </c>
       <c r="K65" t="n">
-        <v>43.17</v>
+        <v>69.81999999999999</v>
       </c>
       <c r="L65" t="n">
-        <v>5.77</v>
+        <v>4.65</v>
       </c>
       <c r="M65" t="n">
-        <v>127.01</v>
+        <v>206.22</v>
       </c>
       <c r="N65" t="inlineStr"/>
       <c r="O65" t="n">
-        <v>9.619999999999999</v>
+        <v>7.75</v>
       </c>
       <c r="P65" t="n">
-        <v>211.68</v>
+        <v>343.7</v>
       </c>
       <c r="Q65" t="inlineStr"/>
       <c r="R65" t="n">
-        <v>19.23</v>
+        <v>15.51</v>
       </c>
       <c r="S65" t="n">
-        <v>423.37</v>
+        <v>687.41</v>
       </c>
       <c r="T65" t="inlineStr"/>
     </row>
@@ -9346,7 +9410,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>SAGA</t>
+          <t>GMT</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -9355,48 +9419,48 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>339939.6</v>
+        <v>325667.9</v>
       </c>
       <c r="E66" t="n">
-        <v>0.01236</v>
+        <v>0.00657</v>
       </c>
       <c r="F66" t="n">
-        <v>0.0126</v>
+        <v>0.00676</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>2026-07-31 17:04</t>
+          <t>2026-07-31 13:55</t>
         </is>
       </c>
       <c r="H66" t="inlineStr"/>
       <c r="I66" t="n">
-        <v>4283.24</v>
+        <v>2201.52</v>
       </c>
       <c r="J66" t="n">
-        <v>1.94</v>
+        <v>2.89</v>
       </c>
       <c r="K66" t="n">
-        <v>83.17</v>
+        <v>63.67</v>
       </c>
       <c r="L66" t="n">
-        <v>5.71</v>
+        <v>8.43</v>
       </c>
       <c r="M66" t="n">
-        <v>244.76</v>
+        <v>185.63</v>
       </c>
       <c r="N66" t="inlineStr"/>
       <c r="O66" t="n">
-        <v>9.52</v>
+        <v>14.05</v>
       </c>
       <c r="P66" t="n">
-        <v>407.93</v>
+        <v>309.38</v>
       </c>
       <c r="Q66" t="inlineStr"/>
       <c r="R66" t="n">
-        <v>19.05</v>
+        <v>28.11</v>
       </c>
       <c r="S66" t="n">
-        <v>815.86</v>
+        <v>618.77</v>
       </c>
       <c r="T66" t="inlineStr"/>
     </row>
@@ -9406,61 +9470,57 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>FLOW</t>
+          <t>SAGA</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>CLOSED</t>
+          <t>OPEN</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>97950.02</v>
+        <v>339939.6</v>
       </c>
       <c r="E67" t="n">
-        <v>0.03081</v>
+        <v>0.01293</v>
       </c>
       <c r="F67" t="n">
-        <v>0.02804405102724839</v>
+        <v>0.0126</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>2026-07-31 17:13</t>
-        </is>
-      </c>
-      <c r="H67" t="inlineStr">
-        <is>
-          <t>2026-07-31 23:28</t>
-        </is>
-      </c>
+          <t>2026-07-31 17:04</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr"/>
       <c r="I67" t="n">
-        <v>2746.92</v>
+        <v>4283.24</v>
       </c>
       <c r="J67" t="n">
-        <v>-8.98</v>
+        <v>-2.55</v>
       </c>
       <c r="K67" t="n">
-        <v>-246.6</v>
+        <v>-109.32</v>
       </c>
       <c r="L67" t="n">
-        <v>-29.59</v>
+        <v>-7.86</v>
       </c>
       <c r="M67" t="n">
-        <v>-812.77</v>
+        <v>-336.54</v>
       </c>
       <c r="N67" t="inlineStr"/>
       <c r="O67" t="n">
-        <v>-49.31</v>
+        <v>-13.1</v>
       </c>
       <c r="P67" t="n">
-        <v>-1354.62</v>
+        <v>-560.9</v>
       </c>
       <c r="Q67" t="inlineStr"/>
       <c r="R67" t="n">
-        <v>-98.63</v>
+        <v>-26.19</v>
       </c>
       <c r="S67" t="n">
-        <v>-2709.25</v>
+        <v>-1121.8</v>
       </c>
       <c r="T67" t="inlineStr"/>
     </row>
@@ -9470,7 +9530,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>TLM</t>
+          <t>FLOW</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -9479,52 +9539,52 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>765466</v>
+        <v>97950.02</v>
       </c>
       <c r="E68" t="n">
-        <v>0.001648650814013947</v>
+        <v>0.03081</v>
       </c>
       <c r="F68" t="n">
-        <v>0.001873560456366487</v>
+        <v>0.02804405102724839</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>2026-08-01 07:57</t>
+          <t>2026-07-31 17:13</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>2026-08-01 10:31</t>
+          <t>2026-07-31 23:28</t>
         </is>
       </c>
       <c r="I68" t="n">
-        <v>1434.15</v>
+        <v>2746.92</v>
       </c>
       <c r="J68" t="n">
-        <v>13.64</v>
+        <v>-8.98</v>
       </c>
       <c r="K68" t="n">
-        <v>195.65</v>
+        <v>-246.6</v>
       </c>
       <c r="L68" t="n">
-        <v>36.01</v>
+        <v>-29.59</v>
       </c>
       <c r="M68" t="n">
-        <v>516.48</v>
+        <v>-812.77</v>
       </c>
       <c r="N68" t="inlineStr"/>
       <c r="O68" t="n">
-        <v>60.02</v>
+        <v>-49.31</v>
       </c>
       <c r="P68" t="n">
-        <v>860.8</v>
+        <v>-1354.62</v>
       </c>
       <c r="Q68" t="inlineStr"/>
       <c r="R68" t="n">
-        <v>120.04</v>
+        <v>-98.63</v>
       </c>
       <c r="S68" t="n">
-        <v>1721.61</v>
+        <v>-2709.25</v>
       </c>
       <c r="T68" t="inlineStr"/>
     </row>
@@ -9543,10 +9603,10 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>382734</v>
+        <v>765466</v>
       </c>
       <c r="E69" t="n">
-        <v>0.001648</v>
+        <v>0.001648650814013947</v>
       </c>
       <c r="F69" t="n">
         <v>0.001873560456366487</v>
@@ -9562,35 +9622,99 @@
         </is>
       </c>
       <c r="I69" t="n">
-        <v>717.08</v>
+        <v>1434.15</v>
       </c>
       <c r="J69" t="n">
-        <v>13.69</v>
+        <v>13.64</v>
       </c>
       <c r="K69" t="n">
-        <v>98.15000000000001</v>
+        <v>195.65</v>
       </c>
       <c r="L69" t="n">
-        <v>36.12</v>
+        <v>36.01</v>
       </c>
       <c r="M69" t="n">
-        <v>258.99</v>
+        <v>516.48</v>
       </c>
       <c r="N69" t="inlineStr"/>
       <c r="O69" t="n">
-        <v>60.2</v>
+        <v>60.02</v>
       </c>
       <c r="P69" t="n">
-        <v>431.65</v>
+        <v>860.8</v>
       </c>
       <c r="Q69" t="inlineStr"/>
       <c r="R69" t="n">
+        <v>120.04</v>
+      </c>
+      <c r="S69" t="n">
+        <v>1721.61</v>
+      </c>
+      <c r="T69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>TLM</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>382734</v>
+      </c>
+      <c r="E70" t="n">
+        <v>0.001648</v>
+      </c>
+      <c r="F70" t="n">
+        <v>0.001873560456366487</v>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>2026-08-01 07:57</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>2026-08-01 10:31</t>
+        </is>
+      </c>
+      <c r="I70" t="n">
+        <v>717.08</v>
+      </c>
+      <c r="J70" t="n">
+        <v>13.69</v>
+      </c>
+      <c r="K70" t="n">
+        <v>98.15000000000001</v>
+      </c>
+      <c r="L70" t="n">
+        <v>36.12</v>
+      </c>
+      <c r="M70" t="n">
+        <v>258.99</v>
+      </c>
+      <c r="N70" t="inlineStr"/>
+      <c r="O70" t="n">
+        <v>60.2</v>
+      </c>
+      <c r="P70" t="n">
+        <v>431.65</v>
+      </c>
+      <c r="Q70" t="inlineStr"/>
+      <c r="R70" t="n">
         <v>120.39</v>
       </c>
-      <c r="S69" t="n">
+      <c r="S70" t="n">
         <v>863.3</v>
       </c>
-      <c r="T69" t="inlineStr"/>
+      <c r="T70" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update trade journal and leverage log (live bot activity)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/leverage_journal.xlsx
+++ b/leverage_journal.xlsx
@@ -459,10 +459,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>106.18</v>
+        <v>186.23</v>
       </c>
       <c r="C2" t="n">
-        <v>47.8</v>
+        <v>47.1</v>
       </c>
       <c r="D2" t="inlineStr"/>
     </row>
@@ -473,10 +473,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2227.31</v>
+        <v>2337.59</v>
       </c>
       <c r="C3" t="n">
-        <v>47.8</v>
+        <v>47.1</v>
       </c>
       <c r="D3" t="n">
         <v>1</v>
@@ -489,10 +489,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4713.47</v>
+        <v>4897.26</v>
       </c>
       <c r="C4" t="n">
-        <v>47.8</v>
+        <v>47.1</v>
       </c>
       <c r="D4" t="n">
         <v>1</v>
@@ -505,10 +505,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>23502.04</v>
+        <v>23869.43</v>
       </c>
       <c r="C5" t="n">
-        <v>47.8</v>
+        <v>47.1</v>
       </c>
       <c r="D5" t="n">
         <v>19</v>
@@ -521,10 +521,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>4937.17</v>
+        <v>4282.67</v>
       </c>
       <c r="C6" t="n">
-        <v>50.7</v>
+        <v>51.4</v>
       </c>
       <c r="D6" t="inlineStr"/>
     </row>
@@ -535,10 +535,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-274.85</v>
+        <v>-515.04</v>
       </c>
       <c r="C7" t="n">
-        <v>50.7</v>
+        <v>51.4</v>
       </c>
       <c r="D7" t="n">
         <v>1</v>
@@ -551,10 +551,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>534.3200000000001</v>
+        <v>134.01</v>
       </c>
       <c r="C8" t="n">
-        <v>52.2</v>
+        <v>52.9</v>
       </c>
       <c r="D8" t="n">
         <v>5</v>
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>12593.43</v>
+        <v>11792.73</v>
       </c>
       <c r="C9" t="n">
-        <v>52.2</v>
+        <v>52.9</v>
       </c>
       <c r="D9" t="n">
         <v>16</v>
@@ -587,7 +587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T70"/>
+  <dimension ref="A1:T71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -713,7 +713,7 @@
         <v>1.589</v>
       </c>
       <c r="F2" t="n">
-        <v>1.434</v>
+        <v>1.468</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -725,30 +725,30 @@
         <v>20.04</v>
       </c>
       <c r="J2" t="n">
-        <v>-9.75</v>
+        <v>-7.61</v>
       </c>
       <c r="K2" t="n">
-        <v>-1.95</v>
+        <v>-1.53</v>
       </c>
       <c r="L2" t="n">
-        <v>-29.26</v>
+        <v>-22.84</v>
       </c>
       <c r="M2" t="n">
-        <v>-5.86</v>
+        <v>-4.58</v>
       </c>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="n">
-        <v>-48.77</v>
+        <v>-38.07</v>
       </c>
       <c r="P2" t="n">
-        <v>-9.77</v>
+        <v>-7.63</v>
       </c>
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="n">
-        <v>-97.55</v>
+        <v>-76.15000000000001</v>
       </c>
       <c r="S2" t="n">
-        <v>-19.55</v>
+        <v>-15.26</v>
       </c>
       <c r="T2" t="inlineStr"/>
     </row>
@@ -773,7 +773,7 @@
         <v>1.588</v>
       </c>
       <c r="F3" t="n">
-        <v>1.434</v>
+        <v>1.468</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -785,30 +785,30 @@
         <v>19.99</v>
       </c>
       <c r="J3" t="n">
-        <v>-9.699999999999999</v>
+        <v>-7.56</v>
       </c>
       <c r="K3" t="n">
-        <v>-1.94</v>
+        <v>-1.51</v>
       </c>
       <c r="L3" t="n">
-        <v>-29.09</v>
+        <v>-22.67</v>
       </c>
       <c r="M3" t="n">
-        <v>-5.81</v>
+        <v>-4.53</v>
       </c>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="n">
-        <v>-48.49</v>
+        <v>-37.78</v>
       </c>
       <c r="P3" t="n">
-        <v>-9.69</v>
+        <v>-7.55</v>
       </c>
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="n">
-        <v>-96.98</v>
+        <v>-75.56999999999999</v>
       </c>
       <c r="S3" t="n">
-        <v>-19.38</v>
+        <v>-15.1</v>
       </c>
       <c r="T3" t="inlineStr"/>
     </row>
@@ -833,7 +833,7 @@
         <v>1.59</v>
       </c>
       <c r="F4" t="n">
-        <v>1.434</v>
+        <v>1.468</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -845,30 +845,30 @@
         <v>20.01</v>
       </c>
       <c r="J4" t="n">
-        <v>-9.81</v>
+        <v>-7.67</v>
       </c>
       <c r="K4" t="n">
-        <v>-1.96</v>
+        <v>-1.54</v>
       </c>
       <c r="L4" t="n">
-        <v>-29.43</v>
+        <v>-23.02</v>
       </c>
       <c r="M4" t="n">
-        <v>-5.89</v>
+        <v>-4.61</v>
       </c>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="n">
-        <v>-49.06</v>
+        <v>-38.36</v>
       </c>
       <c r="P4" t="n">
-        <v>-9.82</v>
+        <v>-7.68</v>
       </c>
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="n">
-        <v>-98.11</v>
+        <v>-76.73</v>
       </c>
       <c r="S4" t="n">
-        <v>-19.63</v>
+        <v>-15.35</v>
       </c>
       <c r="T4" t="inlineStr"/>
     </row>
@@ -2073,7 +2073,7 @@
         <v>2.68</v>
       </c>
       <c r="F23" t="n">
-        <v>2.258</v>
+        <v>2.272</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -2085,23 +2085,23 @@
         <v>5.87</v>
       </c>
       <c r="J23" t="n">
-        <v>-15.75</v>
+        <v>-15.22</v>
       </c>
       <c r="K23" t="n">
-        <v>-0.92</v>
+        <v>-0.89</v>
       </c>
       <c r="L23" t="n">
-        <v>-47.24</v>
+        <v>-45.67</v>
       </c>
       <c r="M23" t="n">
-        <v>-2.77</v>
+        <v>-2.68</v>
       </c>
       <c r="N23" t="inlineStr"/>
       <c r="O23" t="n">
-        <v>-78.73</v>
+        <v>-76.12</v>
       </c>
       <c r="P23" t="n">
-        <v>-4.62</v>
+        <v>-4.47</v>
       </c>
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="n">
@@ -3693,7 +3693,7 @@
         <v>0.1769</v>
       </c>
       <c r="F48" t="n">
-        <v>0.043</v>
+        <v>0.0481</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -3705,10 +3705,10 @@
         <v>1502.06</v>
       </c>
       <c r="J48" t="n">
-        <v>-75.69</v>
+        <v>-72.81</v>
       </c>
       <c r="K48" t="n">
-        <v>-1136.94</v>
+        <v>-1093.64</v>
       </c>
       <c r="L48" t="n">
         <v>-100</v>
@@ -4277,7 +4277,7 @@
         <v>0.01825474902120262</v>
       </c>
       <c r="F57" t="n">
-        <v>0.0191</v>
+        <v>0.01919</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
@@ -4289,30 +4289,30 @@
         <v>2289.31</v>
       </c>
       <c r="J57" t="n">
-        <v>4.63</v>
+        <v>5.12</v>
       </c>
       <c r="K57" t="n">
-        <v>106</v>
+        <v>117.29</v>
       </c>
       <c r="L57" t="n">
-        <v>13.89</v>
+        <v>15.37</v>
       </c>
       <c r="M57" t="n">
-        <v>318.01</v>
+        <v>351.87</v>
       </c>
       <c r="N57" t="inlineStr"/>
       <c r="O57" t="n">
-        <v>23.15</v>
+        <v>25.62</v>
       </c>
       <c r="P57" t="n">
-        <v>530.01</v>
+        <v>586.4400000000001</v>
       </c>
       <c r="Q57" t="inlineStr"/>
       <c r="R57" t="n">
-        <v>46.3</v>
+        <v>51.23</v>
       </c>
       <c r="S57" t="n">
-        <v>1060.02</v>
+        <v>1172.89</v>
       </c>
       <c r="T57" t="inlineStr"/>
     </row>
@@ -4533,7 +4533,7 @@
         <v>0.07548835965087614</v>
       </c>
       <c r="F61" t="n">
-        <v>0.06585000000000001</v>
+        <v>0.06219</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
@@ -4545,23 +4545,23 @@
         <v>0.08</v>
       </c>
       <c r="J61" t="n">
-        <v>-12.77</v>
+        <v>-17.62</v>
       </c>
       <c r="K61" t="n">
         <v>-0.01</v>
       </c>
       <c r="L61" t="n">
-        <v>-38.3</v>
+        <v>-52.85</v>
       </c>
       <c r="M61" t="n">
-        <v>-0.03</v>
+        <v>-0.04</v>
       </c>
       <c r="N61" t="inlineStr"/>
       <c r="O61" t="n">
-        <v>-63.84</v>
+        <v>-88.08</v>
       </c>
       <c r="P61" t="n">
-        <v>-0.05</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="Q61" t="inlineStr"/>
       <c r="R61" t="n">
@@ -4597,7 +4597,7 @@
         <v>0.006940588409461815</v>
       </c>
       <c r="F62" t="n">
-        <v>0.00712</v>
+        <v>0.00711</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
@@ -4609,30 +4609,30 @@
         <v>4538.22</v>
       </c>
       <c r="J62" t="n">
-        <v>2.58</v>
+        <v>2.44</v>
       </c>
       <c r="K62" t="n">
-        <v>117.31</v>
+        <v>110.77</v>
       </c>
       <c r="L62" t="n">
-        <v>7.75</v>
+        <v>7.32</v>
       </c>
       <c r="M62" t="n">
-        <v>351.93</v>
+        <v>332.32</v>
       </c>
       <c r="N62" t="inlineStr"/>
       <c r="O62" t="n">
-        <v>12.92</v>
+        <v>12.2</v>
       </c>
       <c r="P62" t="n">
-        <v>586.5599999999999</v>
+        <v>553.86</v>
       </c>
       <c r="Q62" t="inlineStr"/>
       <c r="R62" t="n">
-        <v>25.85</v>
+        <v>24.41</v>
       </c>
       <c r="S62" t="n">
-        <v>1173.11</v>
+        <v>1107.72</v>
       </c>
       <c r="T62" t="inlineStr"/>
     </row>
@@ -4785,7 +4785,7 @@
         <v>0.04149347287228067</v>
       </c>
       <c r="F65" t="n">
-        <v>0.04085</v>
+        <v>0.03884</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
@@ -4797,30 +4797,30 @@
         <v>4432.66</v>
       </c>
       <c r="J65" t="n">
-        <v>-1.55</v>
+        <v>-6.39</v>
       </c>
       <c r="K65" t="n">
-        <v>-68.73999999999999</v>
+        <v>-283.47</v>
       </c>
       <c r="L65" t="n">
-        <v>-4.65</v>
+        <v>-19.18</v>
       </c>
       <c r="M65" t="n">
-        <v>-206.22</v>
+        <v>-850.4</v>
       </c>
       <c r="N65" t="inlineStr"/>
       <c r="O65" t="n">
-        <v>-7.75</v>
+        <v>-31.97</v>
       </c>
       <c r="P65" t="n">
-        <v>-343.7</v>
+        <v>-1417.33</v>
       </c>
       <c r="Q65" t="inlineStr"/>
       <c r="R65" t="n">
-        <v>-15.51</v>
+        <v>-63.95</v>
       </c>
       <c r="S65" t="n">
-        <v>-687.41</v>
+        <v>-2834.65</v>
       </c>
       <c r="T65" t="inlineStr"/>
     </row>
@@ -4845,7 +4845,7 @@
         <v>0.00676</v>
       </c>
       <c r="F66" t="n">
-        <v>0.00657</v>
+        <v>0.00671</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
@@ -4857,30 +4857,30 @@
         <v>2201.52</v>
       </c>
       <c r="J66" t="n">
-        <v>-2.81</v>
+        <v>-0.74</v>
       </c>
       <c r="K66" t="n">
-        <v>-61.88</v>
+        <v>-16.28</v>
       </c>
       <c r="L66" t="n">
-        <v>-8.43</v>
+        <v>-2.22</v>
       </c>
       <c r="M66" t="n">
-        <v>-185.63</v>
+        <v>-48.85</v>
       </c>
       <c r="N66" t="inlineStr"/>
       <c r="O66" t="n">
-        <v>-14.05</v>
+        <v>-3.7</v>
       </c>
       <c r="P66" t="n">
-        <v>-309.38</v>
+        <v>-81.42</v>
       </c>
       <c r="Q66" t="inlineStr"/>
       <c r="R66" t="n">
-        <v>-28.11</v>
+        <v>-7.4</v>
       </c>
       <c r="S66" t="n">
-        <v>-618.77</v>
+        <v>-162.83</v>
       </c>
       <c r="T66" t="inlineStr"/>
     </row>
@@ -4905,7 +4905,7 @@
         <v>0.0126</v>
       </c>
       <c r="F67" t="n">
-        <v>0.01293</v>
+        <v>0.01356</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
@@ -4917,30 +4917,30 @@
         <v>4283.24</v>
       </c>
       <c r="J67" t="n">
-        <v>2.62</v>
+        <v>7.62</v>
       </c>
       <c r="K67" t="n">
-        <v>112.18</v>
+        <v>326.34</v>
       </c>
       <c r="L67" t="n">
-        <v>7.86</v>
+        <v>22.86</v>
       </c>
       <c r="M67" t="n">
-        <v>336.54</v>
+        <v>979.03</v>
       </c>
       <c r="N67" t="inlineStr"/>
       <c r="O67" t="n">
-        <v>13.1</v>
+        <v>38.1</v>
       </c>
       <c r="P67" t="n">
-        <v>560.9</v>
+        <v>1631.71</v>
       </c>
       <c r="Q67" t="inlineStr"/>
       <c r="R67" t="n">
-        <v>26.19</v>
+        <v>76.19</v>
       </c>
       <c r="S67" t="n">
-        <v>1121.8</v>
+        <v>3263.42</v>
       </c>
       <c r="T67" t="inlineStr"/>
     </row>
@@ -5143,6 +5143,66 @@
           <t>YES</t>
         </is>
       </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>ATM</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>716.3200000000001</v>
+      </c>
+      <c r="E71" t="n">
+        <v>1.613</v>
+      </c>
+      <c r="F71" t="n">
+        <v>1.593</v>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>2026-08-05 09:01</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr"/>
+      <c r="I71" t="n">
+        <v>1155.42</v>
+      </c>
+      <c r="J71" t="n">
+        <v>-1.24</v>
+      </c>
+      <c r="K71" t="n">
+        <v>-14.33</v>
+      </c>
+      <c r="L71" t="n">
+        <v>-3.72</v>
+      </c>
+      <c r="M71" t="n">
+        <v>-42.98</v>
+      </c>
+      <c r="N71" t="inlineStr"/>
+      <c r="O71" t="n">
+        <v>-6.2</v>
+      </c>
+      <c r="P71" t="n">
+        <v>-71.63</v>
+      </c>
+      <c r="Q71" t="inlineStr"/>
+      <c r="R71" t="n">
+        <v>-12.4</v>
+      </c>
+      <c r="S71" t="n">
+        <v>-143.26</v>
+      </c>
+      <c r="T71" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5155,7 +5215,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T70"/>
+  <dimension ref="A1:T71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5278,7 +5338,7 @@
         <v>12.61</v>
       </c>
       <c r="E2" t="n">
-        <v>1.434</v>
+        <v>1.468</v>
       </c>
       <c r="F2" t="n">
         <v>1.589</v>
@@ -5293,30 +5353,30 @@
         <v>20.04</v>
       </c>
       <c r="J2" t="n">
-        <v>10.81</v>
+        <v>8.24</v>
       </c>
       <c r="K2" t="n">
-        <v>2.17</v>
+        <v>1.65</v>
       </c>
       <c r="L2" t="n">
-        <v>29.26</v>
+        <v>22.84</v>
       </c>
       <c r="M2" t="n">
-        <v>5.86</v>
+        <v>4.58</v>
       </c>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="n">
-        <v>48.77</v>
+        <v>38.07</v>
       </c>
       <c r="P2" t="n">
-        <v>9.77</v>
+        <v>7.63</v>
       </c>
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="n">
-        <v>97.55</v>
+        <v>76.15000000000001</v>
       </c>
       <c r="S2" t="n">
-        <v>19.55</v>
+        <v>15.26</v>
       </c>
       <c r="T2" t="inlineStr"/>
     </row>
@@ -5338,7 +5398,7 @@
         <v>12.586</v>
       </c>
       <c r="E3" t="n">
-        <v>1.434</v>
+        <v>1.468</v>
       </c>
       <c r="F3" t="n">
         <v>1.588</v>
@@ -5353,30 +5413,30 @@
         <v>19.99</v>
       </c>
       <c r="J3" t="n">
-        <v>10.74</v>
+        <v>8.17</v>
       </c>
       <c r="K3" t="n">
-        <v>2.15</v>
+        <v>1.63</v>
       </c>
       <c r="L3" t="n">
-        <v>29.09</v>
+        <v>22.67</v>
       </c>
       <c r="M3" t="n">
-        <v>5.81</v>
+        <v>4.53</v>
       </c>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="n">
-        <v>48.49</v>
+        <v>37.78</v>
       </c>
       <c r="P3" t="n">
-        <v>9.69</v>
+        <v>7.55</v>
       </c>
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="n">
-        <v>96.98</v>
+        <v>75.56999999999999</v>
       </c>
       <c r="S3" t="n">
-        <v>19.38</v>
+        <v>15.1</v>
       </c>
       <c r="T3" t="inlineStr"/>
     </row>
@@ -5398,7 +5458,7 @@
         <v>12.586</v>
       </c>
       <c r="E4" t="n">
-        <v>1.434</v>
+        <v>1.468</v>
       </c>
       <c r="F4" t="n">
         <v>1.59</v>
@@ -5413,30 +5473,30 @@
         <v>20.01</v>
       </c>
       <c r="J4" t="n">
-        <v>10.88</v>
+        <v>8.31</v>
       </c>
       <c r="K4" t="n">
-        <v>2.18</v>
+        <v>1.66</v>
       </c>
       <c r="L4" t="n">
-        <v>29.43</v>
+        <v>23.02</v>
       </c>
       <c r="M4" t="n">
-        <v>5.89</v>
+        <v>4.61</v>
       </c>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="n">
-        <v>49.06</v>
+        <v>38.36</v>
       </c>
       <c r="P4" t="n">
-        <v>9.82</v>
+        <v>7.68</v>
       </c>
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="n">
-        <v>98.11</v>
+        <v>76.73</v>
       </c>
       <c r="S4" t="n">
-        <v>19.63</v>
+        <v>15.35</v>
       </c>
       <c r="T4" t="inlineStr"/>
     </row>
@@ -6634,7 +6694,7 @@
         <v>2.19</v>
       </c>
       <c r="E23" t="n">
-        <v>2.258</v>
+        <v>2.272</v>
       </c>
       <c r="F23" t="n">
         <v>2.68</v>
@@ -6649,30 +6709,30 @@
         <v>5.87</v>
       </c>
       <c r="J23" t="n">
-        <v>18.69</v>
+        <v>17.96</v>
       </c>
       <c r="K23" t="n">
-        <v>1.1</v>
+        <v>1.05</v>
       </c>
       <c r="L23" t="n">
-        <v>47.24</v>
+        <v>45.67</v>
       </c>
       <c r="M23" t="n">
-        <v>2.77</v>
+        <v>2.68</v>
       </c>
       <c r="N23" t="inlineStr"/>
       <c r="O23" t="n">
-        <v>78.73</v>
+        <v>76.12</v>
       </c>
       <c r="P23" t="n">
-        <v>4.62</v>
+        <v>4.47</v>
       </c>
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="n">
-        <v>157.46</v>
+        <v>152.24</v>
       </c>
       <c r="S23" t="n">
-        <v>9.24</v>
+        <v>8.94</v>
       </c>
       <c r="T23" t="inlineStr"/>
     </row>
@@ -8258,7 +8318,7 @@
         <v>8491</v>
       </c>
       <c r="E48" t="n">
-        <v>0.043</v>
+        <v>0.0481</v>
       </c>
       <c r="F48" t="n">
         <v>0.1769</v>
@@ -8273,30 +8333,30 @@
         <v>1502.06</v>
       </c>
       <c r="J48" t="n">
-        <v>311.4</v>
+        <v>267.78</v>
       </c>
       <c r="K48" t="n">
-        <v>4677.34</v>
+        <v>4022.14</v>
       </c>
       <c r="L48" t="n">
-        <v>227.08</v>
+        <v>218.43</v>
       </c>
       <c r="M48" t="n">
-        <v>3410.83</v>
+        <v>3280.92</v>
       </c>
       <c r="N48" t="inlineStr"/>
       <c r="O48" t="n">
-        <v>378.46</v>
+        <v>364.05</v>
       </c>
       <c r="P48" t="n">
-        <v>5684.72</v>
+        <v>5468.2</v>
       </c>
       <c r="Q48" t="inlineStr"/>
       <c r="R48" t="n">
-        <v>756.92</v>
+        <v>728.09</v>
       </c>
       <c r="S48" t="n">
-        <v>11369.45</v>
+        <v>10936.41</v>
       </c>
       <c r="T48" t="inlineStr"/>
     </row>
@@ -8842,7 +8902,7 @@
         <v>125409</v>
       </c>
       <c r="E57" t="n">
-        <v>0.0191</v>
+        <v>0.01919</v>
       </c>
       <c r="F57" t="n">
         <v>0.01825474902120262</v>
@@ -8857,30 +8917,30 @@
         <v>2289.31</v>
       </c>
       <c r="J57" t="n">
-        <v>-4.43</v>
+        <v>-4.87</v>
       </c>
       <c r="K57" t="n">
-        <v>-101.31</v>
+        <v>-111.57</v>
       </c>
       <c r="L57" t="n">
-        <v>-13.89</v>
+        <v>-15.37</v>
       </c>
       <c r="M57" t="n">
-        <v>-318.01</v>
+        <v>-351.87</v>
       </c>
       <c r="N57" t="inlineStr"/>
       <c r="O57" t="n">
-        <v>-23.15</v>
+        <v>-25.62</v>
       </c>
       <c r="P57" t="n">
-        <v>-530.01</v>
+        <v>-586.4400000000001</v>
       </c>
       <c r="Q57" t="inlineStr"/>
       <c r="R57" t="n">
-        <v>-46.3</v>
+        <v>-51.23</v>
       </c>
       <c r="S57" t="n">
-        <v>-1060.02</v>
+        <v>-1172.89</v>
       </c>
       <c r="T57" t="inlineStr"/>
     </row>
@@ -9114,7 +9174,7 @@
         <v>1</v>
       </c>
       <c r="E61" t="n">
-        <v>0.06585000000000001</v>
+        <v>0.06219</v>
       </c>
       <c r="F61" t="n">
         <v>0.07548835965087614</v>
@@ -9129,30 +9189,30 @@
         <v>0.08</v>
       </c>
       <c r="J61" t="n">
-        <v>14.64</v>
+        <v>21.38</v>
       </c>
       <c r="K61" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="L61" t="n">
-        <v>38.3</v>
+        <v>52.85</v>
       </c>
       <c r="M61" t="n">
-        <v>0.03</v>
+        <v>0.04</v>
       </c>
       <c r="N61" t="inlineStr"/>
       <c r="O61" t="n">
-        <v>63.84</v>
+        <v>88.08</v>
       </c>
       <c r="P61" t="n">
-        <v>0.05</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="Q61" t="inlineStr"/>
       <c r="R61" t="n">
-        <v>127.68</v>
+        <v>176.16</v>
       </c>
       <c r="S61" t="n">
-        <v>0.1</v>
+        <v>0.13</v>
       </c>
       <c r="T61" t="inlineStr"/>
     </row>
@@ -9174,7 +9234,7 @@
         <v>653866.1</v>
       </c>
       <c r="E62" t="n">
-        <v>0.00712</v>
+        <v>0.00711</v>
       </c>
       <c r="F62" t="n">
         <v>0.006940588409461815</v>
@@ -9189,30 +9249,30 @@
         <v>4538.22</v>
       </c>
       <c r="J62" t="n">
-        <v>-2.52</v>
+        <v>-2.38</v>
       </c>
       <c r="K62" t="n">
-        <v>-114.36</v>
+        <v>-108.13</v>
       </c>
       <c r="L62" t="n">
-        <v>-7.75</v>
+        <v>-7.32</v>
       </c>
       <c r="M62" t="n">
-        <v>-351.93</v>
+        <v>-332.32</v>
       </c>
       <c r="N62" t="inlineStr"/>
       <c r="O62" t="n">
-        <v>-12.92</v>
+        <v>-12.2</v>
       </c>
       <c r="P62" t="n">
-        <v>-586.5599999999999</v>
+        <v>-553.86</v>
       </c>
       <c r="Q62" t="inlineStr"/>
       <c r="R62" t="n">
-        <v>-25.85</v>
+        <v>-24.41</v>
       </c>
       <c r="S62" t="n">
-        <v>-1173.11</v>
+        <v>-1107.72</v>
       </c>
       <c r="T62" t="inlineStr"/>
     </row>
@@ -9362,7 +9422,7 @@
         <v>106828</v>
       </c>
       <c r="E65" t="n">
-        <v>0.04085</v>
+        <v>0.03884</v>
       </c>
       <c r="F65" t="n">
         <v>0.04149347287228067</v>
@@ -9377,30 +9437,30 @@
         <v>4432.66</v>
       </c>
       <c r="J65" t="n">
-        <v>1.58</v>
+        <v>6.83</v>
       </c>
       <c r="K65" t="n">
-        <v>69.81999999999999</v>
+        <v>302.83</v>
       </c>
       <c r="L65" t="n">
-        <v>4.65</v>
+        <v>19.18</v>
       </c>
       <c r="M65" t="n">
-        <v>206.22</v>
+        <v>850.4</v>
       </c>
       <c r="N65" t="inlineStr"/>
       <c r="O65" t="n">
-        <v>7.75</v>
+        <v>31.97</v>
       </c>
       <c r="P65" t="n">
-        <v>343.7</v>
+        <v>1417.33</v>
       </c>
       <c r="Q65" t="inlineStr"/>
       <c r="R65" t="n">
-        <v>15.51</v>
+        <v>63.95</v>
       </c>
       <c r="S65" t="n">
-        <v>687.41</v>
+        <v>2834.65</v>
       </c>
       <c r="T65" t="inlineStr"/>
     </row>
@@ -9422,7 +9482,7 @@
         <v>325667.9</v>
       </c>
       <c r="E66" t="n">
-        <v>0.00657</v>
+        <v>0.00671</v>
       </c>
       <c r="F66" t="n">
         <v>0.00676</v>
@@ -9437,30 +9497,30 @@
         <v>2201.52</v>
       </c>
       <c r="J66" t="n">
-        <v>2.89</v>
+        <v>0.75</v>
       </c>
       <c r="K66" t="n">
-        <v>63.67</v>
+        <v>16.4</v>
       </c>
       <c r="L66" t="n">
-        <v>8.43</v>
+        <v>2.22</v>
       </c>
       <c r="M66" t="n">
-        <v>185.63</v>
+        <v>48.85</v>
       </c>
       <c r="N66" t="inlineStr"/>
       <c r="O66" t="n">
-        <v>14.05</v>
+        <v>3.7</v>
       </c>
       <c r="P66" t="n">
-        <v>309.38</v>
+        <v>81.42</v>
       </c>
       <c r="Q66" t="inlineStr"/>
       <c r="R66" t="n">
-        <v>28.11</v>
+        <v>7.4</v>
       </c>
       <c r="S66" t="n">
-        <v>618.77</v>
+        <v>162.83</v>
       </c>
       <c r="T66" t="inlineStr"/>
     </row>
@@ -9482,7 +9542,7 @@
         <v>339939.6</v>
       </c>
       <c r="E67" t="n">
-        <v>0.01293</v>
+        <v>0.01356</v>
       </c>
       <c r="F67" t="n">
         <v>0.0126</v>
@@ -9497,30 +9557,30 @@
         <v>4283.24</v>
       </c>
       <c r="J67" t="n">
-        <v>-2.55</v>
+        <v>-7.08</v>
       </c>
       <c r="K67" t="n">
-        <v>-109.32</v>
+        <v>-303.24</v>
       </c>
       <c r="L67" t="n">
-        <v>-7.86</v>
+        <v>-22.86</v>
       </c>
       <c r="M67" t="n">
-        <v>-336.54</v>
+        <v>-979.03</v>
       </c>
       <c r="N67" t="inlineStr"/>
       <c r="O67" t="n">
-        <v>-13.1</v>
+        <v>-38.1</v>
       </c>
       <c r="P67" t="n">
-        <v>-560.9</v>
+        <v>-1631.71</v>
       </c>
       <c r="Q67" t="inlineStr"/>
       <c r="R67" t="n">
-        <v>-26.19</v>
+        <v>-76.19</v>
       </c>
       <c r="S67" t="n">
-        <v>-1121.8</v>
+        <v>-3263.42</v>
       </c>
       <c r="T67" t="inlineStr"/>
     </row>
@@ -9715,6 +9775,66 @@
         <v>863.3</v>
       </c>
       <c r="T70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>ATM</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>716.3200000000001</v>
+      </c>
+      <c r="E71" t="n">
+        <v>1.593</v>
+      </c>
+      <c r="F71" t="n">
+        <v>1.613</v>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>2026-08-05 09:01</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr"/>
+      <c r="I71" t="n">
+        <v>1155.42</v>
+      </c>
+      <c r="J71" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="K71" t="n">
+        <v>14.51</v>
+      </c>
+      <c r="L71" t="n">
+        <v>3.72</v>
+      </c>
+      <c r="M71" t="n">
+        <v>42.98</v>
+      </c>
+      <c r="N71" t="inlineStr"/>
+      <c r="O71" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="P71" t="n">
+        <v>71.63</v>
+      </c>
+      <c r="Q71" t="inlineStr"/>
+      <c r="R71" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="S71" t="n">
+        <v>143.26</v>
+      </c>
+      <c r="T71" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>